<commit_message>
tg done not full
</commit_message>
<xml_diff>
--- a/1. Почасовая выручка (Отчет инсайда) 02.10.2026 15.12.07.xlsx
+++ b/1. Почасовая выручка (Отчет инсайда) 02.10.2026 15.12.07.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/inkonio/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/inkonio/Desktop/im 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F912A137-0FF1-8A42-BDC6-D63E35460FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44201ADF-50B8-674F-A0A2-CD8EFCBCB050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -290,7 +290,13 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -299,13 +305,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -605,42 +605,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -658,10 +658,10 @@
       <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="13"/>
+      <c r="G5" s="10"/>
     </row>
     <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -679,14 +679,14 @@
       <c r="E6" s="6">
         <v>3150</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="11">
         <v>3150</v>
       </c>
-      <c r="G6" s="9"/>
+      <c r="G6" s="11"/>
     </row>
     <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="1" t="s">
         <v>12</v>
       </c>
@@ -696,14 +696,14 @@
       <c r="E7" s="6">
         <v>22120</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="11">
         <v>3160</v>
       </c>
-      <c r="G7" s="9"/>
+      <c r="G7" s="11"/>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="1" t="s">
         <v>13</v>
       </c>
@@ -713,14 +713,14 @@
       <c r="E8" s="6">
         <v>67300</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="11">
         <v>3502.32</v>
       </c>
-      <c r="G8" s="9"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
@@ -730,14 +730,14 @@
       <c r="E9" s="6">
         <v>108350</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="11">
         <v>3009.72</v>
       </c>
-      <c r="G9" s="9"/>
+      <c r="G9" s="11"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
@@ -747,14 +747,14 @@
       <c r="E10" s="6">
         <v>163920</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="11">
         <v>3092.83</v>
       </c>
-      <c r="G10" s="9"/>
+      <c r="G10" s="11"/>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="1" t="s">
         <v>16</v>
       </c>
@@ -764,14 +764,14 @@
       <c r="E11" s="6">
         <v>175430</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="11">
         <v>3439.8</v>
       </c>
-      <c r="G11" s="9"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="1" t="s">
         <v>17</v>
       </c>
@@ -781,14 +781,14 @@
       <c r="E12" s="6">
         <v>170250</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="11">
         <v>3622.34</v>
       </c>
-      <c r="G12" s="9"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
@@ -798,14 +798,14 @@
       <c r="E13" s="6">
         <v>120450</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="11">
         <v>3345.83</v>
       </c>
-      <c r="G13" s="9"/>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="1" t="s">
         <v>19</v>
       </c>
@@ -815,14 +815,14 @@
       <c r="E14" s="6">
         <v>144250</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="11">
         <v>4371.21</v>
       </c>
-      <c r="G14" s="9"/>
+      <c r="G14" s="11"/>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
       <c r="C15" s="1" t="s">
         <v>20</v>
       </c>
@@ -832,14 +832,14 @@
       <c r="E15" s="6">
         <v>151400</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="11">
         <v>4684</v>
       </c>
-      <c r="G15" s="9"/>
+      <c r="G15" s="11"/>
     </row>
     <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
       <c r="C16" s="1" t="s">
         <v>21</v>
       </c>
@@ -849,14 +849,14 @@
       <c r="E16" s="6">
         <v>60200</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="11">
         <v>3962.93</v>
       </c>
-      <c r="G16" s="9"/>
+      <c r="G16" s="11"/>
     </row>
     <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="1" t="s">
         <v>22</v>
       </c>
@@ -866,14 +866,14 @@
       <c r="E17" s="6">
         <v>330500</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="11">
         <v>4070.91</v>
       </c>
-      <c r="G17" s="9"/>
+      <c r="G17" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
       <c r="C18" s="1" t="s">
         <v>23</v>
       </c>
@@ -883,14 +883,14 @@
       <c r="E18" s="6">
         <v>107250</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="11">
         <v>3972.22</v>
       </c>
-      <c r="G18" s="9"/>
+      <c r="G18" s="11"/>
     </row>
     <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="1" t="s">
         <v>24</v>
       </c>
@@ -900,14 +900,14 @@
       <c r="E19" s="6">
         <v>73250</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="11">
         <v>4832.93</v>
       </c>
-      <c r="G19" s="9"/>
+      <c r="G19" s="11"/>
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
       <c r="C20" s="1" t="s">
         <v>25</v>
       </c>
@@ -917,30 +917,30 @@
       <c r="E20" s="6">
         <v>68270</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="11">
         <v>5458.5</v>
       </c>
-      <c r="G20" s="9"/>
+      <c r="G20" s="11"/>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10"/>
-      <c r="B21" s="8" t="s">
+      <c r="A21" s="12"/>
+      <c r="B21" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="8"/>
+      <c r="C21" s="13"/>
       <c r="D21" s="5">
         <v>463</v>
       </c>
       <c r="E21" s="6">
         <v>1766090</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="11">
         <v>3782.34</v>
       </c>
-      <c r="G21" s="9"/>
+      <c r="G21" s="11"/>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10"/>
+      <c r="A22" s="12"/>
       <c r="B22" s="4">
         <v>46280</v>
       </c>
@@ -953,14 +953,14 @@
       <c r="E22" s="6">
         <v>3850</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="11">
         <v>1283.33</v>
       </c>
-      <c r="G22" s="9"/>
+      <c r="G22" s="11"/>
     </row>
     <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="1" t="s">
         <v>12</v>
       </c>
@@ -970,14 +970,14 @@
       <c r="E23" s="6">
         <v>12650</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="11">
         <v>3162.5</v>
       </c>
-      <c r="G23" s="9"/>
+      <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
       <c r="C24" s="1" t="s">
         <v>13</v>
       </c>
@@ -987,14 +987,14 @@
       <c r="E24" s="6">
         <v>36900</v>
       </c>
-      <c r="F24" s="9">
+      <c r="F24" s="11">
         <v>3690</v>
       </c>
-      <c r="G24" s="9"/>
+      <c r="G24" s="11"/>
     </row>
     <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="1" t="s">
         <v>14</v>
       </c>
@@ -1004,14 +1004,14 @@
       <c r="E25" s="6">
         <v>175730</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="11">
         <v>3430.86</v>
       </c>
-      <c r="G25" s="9"/>
+      <c r="G25" s="11"/>
     </row>
     <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
@@ -1021,14 +1021,14 @@
       <c r="E26" s="6">
         <v>188850</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="11">
         <v>2985.62</v>
       </c>
-      <c r="G26" s="9"/>
+      <c r="G26" s="11"/>
     </row>
     <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="1" t="s">
         <v>16</v>
       </c>
@@ -1038,14 +1038,14 @@
       <c r="E27" s="6">
         <v>151650</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="11">
         <v>3064.04</v>
       </c>
-      <c r="G27" s="9"/>
+      <c r="G27" s="11"/>
     </row>
     <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
       <c r="C28" s="1" t="s">
         <v>17</v>
       </c>
@@ -1055,14 +1055,14 @@
       <c r="E28" s="6">
         <v>149570</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F28" s="11">
         <v>3382.14</v>
       </c>
-      <c r="G28" s="9"/>
+      <c r="G28" s="11"/>
     </row>
     <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
       <c r="C29" s="1" t="s">
         <v>18</v>
       </c>
@@ -1072,14 +1072,14 @@
       <c r="E29" s="6">
         <v>231710</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="11">
         <v>3861.83</v>
       </c>
-      <c r="G29" s="9"/>
+      <c r="G29" s="11"/>
     </row>
     <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
       <c r="C30" s="1" t="s">
         <v>19</v>
       </c>
@@ -1089,14 +1089,14 @@
       <c r="E30" s="6">
         <v>155600</v>
       </c>
-      <c r="F30" s="9">
+      <c r="F30" s="11">
         <v>4184.97</v>
       </c>
-      <c r="G30" s="9"/>
+      <c r="G30" s="11"/>
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
       <c r="C31" s="1" t="s">
         <v>20</v>
       </c>
@@ -1106,14 +1106,14 @@
       <c r="E31" s="6">
         <v>195350</v>
       </c>
-      <c r="F31" s="9">
+      <c r="F31" s="11">
         <v>4422.59</v>
       </c>
-      <c r="G31" s="9"/>
+      <c r="G31" s="11"/>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
+      <c r="A32" s="12"/>
+      <c r="B32" s="12"/>
       <c r="C32" s="1" t="s">
         <v>21</v>
       </c>
@@ -1123,14 +1123,14 @@
       <c r="E32" s="6">
         <v>236710</v>
       </c>
-      <c r="F32" s="9">
+      <c r="F32" s="11">
         <v>3641.69</v>
       </c>
-      <c r="G32" s="9"/>
+      <c r="G32" s="11"/>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="1" t="s">
         <v>22</v>
       </c>
@@ -1140,14 +1140,14 @@
       <c r="E33" s="6">
         <v>136250</v>
       </c>
-      <c r="F33" s="9">
+      <c r="F33" s="11">
         <v>3168.6</v>
       </c>
-      <c r="G33" s="9"/>
+      <c r="G33" s="11"/>
     </row>
     <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
+      <c r="A34" s="12"/>
+      <c r="B34" s="12"/>
       <c r="C34" s="1" t="s">
         <v>23</v>
       </c>
@@ -1157,14 +1157,14 @@
       <c r="E34" s="6">
         <v>102900</v>
       </c>
-      <c r="F34" s="9">
+      <c r="F34" s="11">
         <v>3118.18</v>
       </c>
-      <c r="G34" s="9"/>
+      <c r="G34" s="11"/>
     </row>
     <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
       <c r="C35" s="1" t="s">
         <v>24</v>
       </c>
@@ -1174,14 +1174,14 @@
       <c r="E35" s="6">
         <v>74150</v>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="11">
         <v>3089.58</v>
       </c>
-      <c r="G35" s="9"/>
+      <c r="G35" s="11"/>
     </row>
     <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
       <c r="C36" s="1" t="s">
         <v>25</v>
       </c>
@@ -1191,30 +1191,30 @@
       <c r="E36" s="6">
         <v>22850</v>
       </c>
-      <c r="F36" s="9">
+      <c r="F36" s="11">
         <v>5712.5</v>
       </c>
-      <c r="G36" s="9"/>
+      <c r="G36" s="11"/>
     </row>
     <row r="37" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="8" t="s">
+      <c r="A37" s="12"/>
+      <c r="B37" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="8"/>
+      <c r="C37" s="13"/>
       <c r="D37" s="5">
         <v>534</v>
       </c>
       <c r="E37" s="6">
         <v>1874720</v>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="11">
         <v>3500.8</v>
       </c>
-      <c r="G37" s="9"/>
+      <c r="G37" s="11"/>
     </row>
     <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="10"/>
+      <c r="A38" s="12"/>
       <c r="B38" s="4">
         <v>46281</v>
       </c>
@@ -1227,14 +1227,14 @@
       <c r="E38" s="6">
         <v>9100</v>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="11">
         <v>3033.33</v>
       </c>
-      <c r="G38" s="9"/>
+      <c r="G38" s="11"/>
     </row>
     <row r="39" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
       <c r="C39" s="1" t="s">
         <v>12</v>
       </c>
@@ -1244,14 +1244,14 @@
       <c r="E39" s="6">
         <v>17450</v>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="11">
         <v>2492.86</v>
       </c>
-      <c r="G39" s="9"/>
+      <c r="G39" s="11"/>
     </row>
     <row r="40" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10"/>
+      <c r="A40" s="12"/>
+      <c r="B40" s="12"/>
       <c r="C40" s="1" t="s">
         <v>13</v>
       </c>
@@ -1261,14 +1261,14 @@
       <c r="E40" s="6">
         <v>30650</v>
       </c>
-      <c r="F40" s="9">
+      <c r="F40" s="11">
         <v>3065</v>
       </c>
-      <c r="G40" s="9"/>
+      <c r="G40" s="11"/>
     </row>
     <row r="41" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
       <c r="C41" s="1" t="s">
         <v>14</v>
       </c>
@@ -1278,14 +1278,14 @@
       <c r="E41" s="6">
         <v>98450</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="11">
         <v>3516.07</v>
       </c>
-      <c r="G41" s="9"/>
+      <c r="G41" s="11"/>
     </row>
     <row r="42" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
       <c r="C42" s="1" t="s">
         <v>15</v>
       </c>
@@ -1295,14 +1295,14 @@
       <c r="E42" s="6">
         <v>131010</v>
       </c>
-      <c r="F42" s="9">
+      <c r="F42" s="11">
         <v>3639.17</v>
       </c>
-      <c r="G42" s="9"/>
+      <c r="G42" s="11"/>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
       <c r="C43" s="1" t="s">
         <v>16</v>
       </c>
@@ -1312,14 +1312,14 @@
       <c r="E43" s="6">
         <v>99050</v>
       </c>
-      <c r="F43" s="9">
+      <c r="F43" s="11">
         <v>2677.03</v>
       </c>
-      <c r="G43" s="9"/>
+      <c r="G43" s="11"/>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="10"/>
-      <c r="B44" s="10"/>
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
       <c r="C44" s="1" t="s">
         <v>17</v>
       </c>
@@ -1329,14 +1329,14 @@
       <c r="E44" s="6">
         <v>86770</v>
       </c>
-      <c r="F44" s="9">
+      <c r="F44" s="11">
         <v>2799.03</v>
       </c>
-      <c r="G44" s="9"/>
+      <c r="G44" s="11"/>
     </row>
     <row r="45" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10"/>
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
       <c r="C45" s="1" t="s">
         <v>18</v>
       </c>
@@ -1346,14 +1346,14 @@
       <c r="E45" s="6">
         <v>94750</v>
       </c>
-      <c r="F45" s="9">
+      <c r="F45" s="11">
         <v>3644.23</v>
       </c>
-      <c r="G45" s="9"/>
+      <c r="G45" s="11"/>
     </row>
     <row r="46" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10"/>
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
       <c r="C46" s="1" t="s">
         <v>19</v>
       </c>
@@ -1363,14 +1363,14 @@
       <c r="E46" s="6">
         <v>101350</v>
       </c>
-      <c r="F46" s="9">
+      <c r="F46" s="11">
         <v>2895.71</v>
       </c>
-      <c r="G46" s="9"/>
+      <c r="G46" s="11"/>
     </row>
     <row r="47" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10"/>
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
       <c r="C47" s="1" t="s">
         <v>20</v>
       </c>
@@ -1380,14 +1380,14 @@
       <c r="E47" s="6">
         <v>178350</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="11">
         <v>4147.67</v>
       </c>
-      <c r="G47" s="9"/>
+      <c r="G47" s="11"/>
     </row>
     <row r="48" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="10"/>
-      <c r="B48" s="10"/>
+      <c r="A48" s="12"/>
+      <c r="B48" s="12"/>
       <c r="C48" s="1" t="s">
         <v>21</v>
       </c>
@@ -1397,14 +1397,14 @@
       <c r="E48" s="6">
         <v>149720</v>
       </c>
-      <c r="F48" s="9">
+      <c r="F48" s="11">
         <v>2935.69</v>
       </c>
-      <c r="G48" s="9"/>
+      <c r="G48" s="11"/>
     </row>
     <row r="49" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="10"/>
-      <c r="B49" s="10"/>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
       <c r="C49" s="1" t="s">
         <v>22</v>
       </c>
@@ -1414,14 +1414,14 @@
       <c r="E49" s="6">
         <v>133110</v>
       </c>
-      <c r="F49" s="9">
+      <c r="F49" s="11">
         <v>3502.89</v>
       </c>
-      <c r="G49" s="9"/>
+      <c r="G49" s="11"/>
     </row>
     <row r="50" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
       <c r="C50" s="1" t="s">
         <v>23</v>
       </c>
@@ -1431,14 +1431,14 @@
       <c r="E50" s="6">
         <v>147550</v>
       </c>
-      <c r="F50" s="9">
+      <c r="F50" s="11">
         <v>3353.41</v>
       </c>
-      <c r="G50" s="9"/>
+      <c r="G50" s="11"/>
     </row>
     <row r="51" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="10"/>
-      <c r="B51" s="10"/>
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
       <c r="C51" s="1" t="s">
         <v>24</v>
       </c>
@@ -1448,14 +1448,14 @@
       <c r="E51" s="6">
         <v>50850</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="11">
         <v>2311.36</v>
       </c>
-      <c r="G51" s="9"/>
+      <c r="G51" s="11"/>
     </row>
     <row r="52" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="10"/>
-      <c r="B52" s="10"/>
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
       <c r="C52" s="1" t="s">
         <v>25</v>
       </c>
@@ -1465,30 +1465,31 @@
       <c r="E52" s="6">
         <v>6700</v>
       </c>
-      <c r="F52" s="9">
+      <c r="F52" s="11">
         <v>3350</v>
       </c>
-      <c r="G52" s="9"/>
+      <c r="G52" s="11"/>
     </row>
     <row r="53" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="10"/>
-      <c r="B53" s="8" t="s">
+      <c r="A53" s="12"/>
+      <c r="B53" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C53" s="8"/>
+      <c r="C53" s="13"/>
       <c r="D53" s="5">
+        <f>SUM(D38:D52)</f>
         <v>413</v>
       </c>
       <c r="E53" s="6">
         <v>1334860</v>
       </c>
-      <c r="F53" s="9">
+      <c r="F53" s="11">
         <v>3232.11</v>
       </c>
-      <c r="G53" s="9"/>
+      <c r="G53" s="11"/>
     </row>
     <row r="54" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="10"/>
+      <c r="A54" s="12"/>
       <c r="B54" s="4">
         <v>46282</v>
       </c>
@@ -1501,14 +1502,14 @@
       <c r="E54" s="6">
         <v>1100</v>
       </c>
-      <c r="F54" s="9">
+      <c r="F54" s="11">
         <v>1100</v>
       </c>
-      <c r="G54" s="9"/>
+      <c r="G54" s="11"/>
     </row>
     <row r="55" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="10"/>
-      <c r="B55" s="10"/>
+      <c r="A55" s="12"/>
+      <c r="B55" s="12"/>
       <c r="C55" s="1" t="s">
         <v>12</v>
       </c>
@@ -1518,14 +1519,14 @@
       <c r="E55" s="6">
         <v>4150</v>
       </c>
-      <c r="F55" s="9">
+      <c r="F55" s="11">
         <v>2075</v>
       </c>
-      <c r="G55" s="9"/>
+      <c r="G55" s="11"/>
     </row>
     <row r="56" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="10"/>
-      <c r="B56" s="10"/>
+      <c r="A56" s="12"/>
+      <c r="B56" s="12"/>
       <c r="C56" s="1" t="s">
         <v>13</v>
       </c>
@@ -1535,14 +1536,14 @@
       <c r="E56" s="6">
         <v>23750</v>
       </c>
-      <c r="F56" s="9">
+      <c r="F56" s="11">
         <v>2638.89</v>
       </c>
-      <c r="G56" s="9"/>
+      <c r="G56" s="11"/>
     </row>
     <row r="57" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
+      <c r="A57" s="12"/>
+      <c r="B57" s="12"/>
       <c r="C57" s="1" t="s">
         <v>14</v>
       </c>
@@ -1552,14 +1553,14 @@
       <c r="E57" s="6">
         <v>99250</v>
       </c>
-      <c r="F57" s="9">
+      <c r="F57" s="11">
         <v>2835.71</v>
       </c>
-      <c r="G57" s="9"/>
+      <c r="G57" s="11"/>
     </row>
     <row r="58" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10"/>
-      <c r="B58" s="10"/>
+      <c r="A58" s="12"/>
+      <c r="B58" s="12"/>
       <c r="C58" s="1" t="s">
         <v>15</v>
       </c>
@@ -1569,14 +1570,14 @@
       <c r="E58" s="6">
         <v>173100</v>
       </c>
-      <c r="F58" s="9">
+      <c r="F58" s="11">
         <v>2933.9</v>
       </c>
-      <c r="G58" s="9"/>
+      <c r="G58" s="11"/>
     </row>
     <row r="59" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="10"/>
-      <c r="B59" s="10"/>
+      <c r="A59" s="12"/>
+      <c r="B59" s="12"/>
       <c r="C59" s="1" t="s">
         <v>16</v>
       </c>
@@ -1586,14 +1587,14 @@
       <c r="E59" s="6">
         <v>116450</v>
       </c>
-      <c r="F59" s="9">
+      <c r="F59" s="11">
         <v>3756.45</v>
       </c>
-      <c r="G59" s="9"/>
+      <c r="G59" s="11"/>
     </row>
     <row r="60" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="10"/>
-      <c r="B60" s="10"/>
+      <c r="A60" s="12"/>
+      <c r="B60" s="12"/>
       <c r="C60" s="1" t="s">
         <v>17</v>
       </c>
@@ -1603,14 +1604,14 @@
       <c r="E60" s="6">
         <v>94600</v>
       </c>
-      <c r="F60" s="9">
+      <c r="F60" s="11">
         <v>3503.7</v>
       </c>
-      <c r="G60" s="9"/>
+      <c r="G60" s="11"/>
     </row>
     <row r="61" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10"/>
-      <c r="B61" s="10"/>
+      <c r="A61" s="12"/>
+      <c r="B61" s="12"/>
       <c r="C61" s="1" t="s">
         <v>18</v>
       </c>
@@ -1620,14 +1621,14 @@
       <c r="E61" s="6">
         <v>124850</v>
       </c>
-      <c r="F61" s="9">
+      <c r="F61" s="11">
         <v>4161.67</v>
       </c>
-      <c r="G61" s="9"/>
+      <c r="G61" s="11"/>
     </row>
     <row r="62" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="10"/>
-      <c r="B62" s="10"/>
+      <c r="A62" s="12"/>
+      <c r="B62" s="12"/>
       <c r="C62" s="1" t="s">
         <v>19</v>
       </c>
@@ -1637,14 +1638,14 @@
       <c r="E62" s="6">
         <v>119950</v>
       </c>
-      <c r="F62" s="9">
+      <c r="F62" s="11">
         <v>3634.85</v>
       </c>
-      <c r="G62" s="9"/>
+      <c r="G62" s="11"/>
     </row>
     <row r="63" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="10"/>
-      <c r="B63" s="10"/>
+      <c r="A63" s="12"/>
+      <c r="B63" s="12"/>
       <c r="C63" s="1" t="s">
         <v>20</v>
       </c>
@@ -1654,14 +1655,14 @@
       <c r="E63" s="6">
         <v>184910</v>
       </c>
-      <c r="F63" s="9">
+      <c r="F63" s="11">
         <v>3555.96</v>
       </c>
-      <c r="G63" s="9"/>
+      <c r="G63" s="11"/>
     </row>
     <row r="64" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="10"/>
-      <c r="B64" s="10"/>
+      <c r="A64" s="12"/>
+      <c r="B64" s="12"/>
       <c r="C64" s="1" t="s">
         <v>21</v>
       </c>
@@ -1671,14 +1672,14 @@
       <c r="E64" s="6">
         <v>144960</v>
       </c>
-      <c r="F64" s="9">
+      <c r="F64" s="11">
         <v>3084.26</v>
       </c>
-      <c r="G64" s="9"/>
+      <c r="G64" s="11"/>
     </row>
     <row r="65" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="10"/>
-      <c r="B65" s="10"/>
+      <c r="A65" s="12"/>
+      <c r="B65" s="12"/>
       <c r="C65" s="1" t="s">
         <v>22</v>
       </c>
@@ -1688,14 +1689,14 @@
       <c r="E65" s="6">
         <v>211920</v>
       </c>
-      <c r="F65" s="9">
+      <c r="F65" s="11">
         <v>3653.79</v>
       </c>
-      <c r="G65" s="9"/>
+      <c r="G65" s="11"/>
     </row>
     <row r="66" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="10"/>
-      <c r="B66" s="10"/>
+      <c r="A66" s="12"/>
+      <c r="B66" s="12"/>
       <c r="C66" s="1" t="s">
         <v>23</v>
       </c>
@@ -1705,14 +1706,14 @@
       <c r="E66" s="6">
         <v>60910</v>
       </c>
-      <c r="F66" s="9">
+      <c r="F66" s="11">
         <v>2768.64</v>
       </c>
-      <c r="G66" s="9"/>
+      <c r="G66" s="11"/>
     </row>
     <row r="67" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="10"/>
-      <c r="B67" s="10"/>
+      <c r="A67" s="12"/>
+      <c r="B67" s="12"/>
       <c r="C67" s="1" t="s">
         <v>24</v>
       </c>
@@ -1722,14 +1723,14 @@
       <c r="E67" s="6">
         <v>52900</v>
       </c>
-      <c r="F67" s="9">
+      <c r="F67" s="11">
         <v>3306.25</v>
       </c>
-      <c r="G67" s="9"/>
+      <c r="G67" s="11"/>
     </row>
     <row r="68" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
+      <c r="A68" s="12"/>
+      <c r="B68" s="12"/>
       <c r="C68" s="1" t="s">
         <v>25</v>
       </c>
@@ -1739,30 +1740,30 @@
       <c r="E68" s="6">
         <v>26700</v>
       </c>
-      <c r="F68" s="9">
+      <c r="F68" s="11">
         <v>4450</v>
       </c>
-      <c r="G68" s="9"/>
+      <c r="G68" s="11"/>
     </row>
     <row r="69" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="10"/>
-      <c r="B69" s="8" t="s">
+      <c r="A69" s="12"/>
+      <c r="B69" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C69" s="8"/>
+      <c r="C69" s="13"/>
       <c r="D69" s="5">
         <v>428</v>
       </c>
       <c r="E69" s="6">
         <v>1439500</v>
       </c>
-      <c r="F69" s="9">
+      <c r="F69" s="11">
         <v>3363.32</v>
       </c>
-      <c r="G69" s="9"/>
+      <c r="G69" s="11"/>
     </row>
     <row r="70" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="10"/>
+      <c r="A70" s="12"/>
       <c r="B70" s="4">
         <v>46283</v>
       </c>
@@ -1775,14 +1776,14 @@
       <c r="E70" s="6">
         <v>10</v>
       </c>
-      <c r="F70" s="9">
+      <c r="F70" s="11">
         <v>10</v>
       </c>
-      <c r="G70" s="9"/>
+      <c r="G70" s="11"/>
     </row>
     <row r="71" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="10"/>
-      <c r="B71" s="10"/>
+      <c r="A71" s="12"/>
+      <c r="B71" s="12"/>
       <c r="C71" s="1" t="s">
         <v>12</v>
       </c>
@@ -1792,14 +1793,14 @@
       <c r="E71" s="6">
         <v>10350</v>
       </c>
-      <c r="F71" s="9">
+      <c r="F71" s="11">
         <v>2587.5</v>
       </c>
-      <c r="G71" s="9"/>
+      <c r="G71" s="11"/>
     </row>
     <row r="72" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="10"/>
-      <c r="B72" s="10"/>
+      <c r="A72" s="12"/>
+      <c r="B72" s="12"/>
       <c r="C72" s="1" t="s">
         <v>13</v>
       </c>
@@ -1809,14 +1810,14 @@
       <c r="E72" s="6">
         <v>29400</v>
       </c>
-      <c r="F72" s="9">
+      <c r="F72" s="11">
         <v>3266.67</v>
       </c>
-      <c r="G72" s="9"/>
+      <c r="G72" s="11"/>
     </row>
     <row r="73" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="10"/>
-      <c r="B73" s="10"/>
+      <c r="A73" s="12"/>
+      <c r="B73" s="12"/>
       <c r="C73" s="1" t="s">
         <v>14</v>
       </c>
@@ -1826,14 +1827,14 @@
       <c r="E73" s="6">
         <v>102300</v>
       </c>
-      <c r="F73" s="9">
+      <c r="F73" s="11">
         <v>3653.57</v>
       </c>
-      <c r="G73" s="9"/>
+      <c r="G73" s="11"/>
     </row>
     <row r="74" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="10"/>
-      <c r="B74" s="10"/>
+      <c r="A74" s="12"/>
+      <c r="B74" s="12"/>
       <c r="C74" s="1" t="s">
         <v>15</v>
       </c>
@@ -1843,14 +1844,14 @@
       <c r="E74" s="6">
         <v>189690</v>
       </c>
-      <c r="F74" s="9">
+      <c r="F74" s="11">
         <v>3010.95</v>
       </c>
-      <c r="G74" s="9"/>
+      <c r="G74" s="11"/>
     </row>
     <row r="75" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="10"/>
-      <c r="B75" s="10"/>
+      <c r="A75" s="12"/>
+      <c r="B75" s="12"/>
       <c r="C75" s="1" t="s">
         <v>16</v>
       </c>
@@ -1860,14 +1861,14 @@
       <c r="E75" s="6">
         <v>170800</v>
       </c>
-      <c r="F75" s="9">
+      <c r="F75" s="11">
         <v>3162.96</v>
       </c>
-      <c r="G75" s="9"/>
+      <c r="G75" s="11"/>
     </row>
     <row r="76" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="10"/>
-      <c r="B76" s="10"/>
+      <c r="A76" s="12"/>
+      <c r="B76" s="12"/>
       <c r="C76" s="1" t="s">
         <v>17</v>
       </c>
@@ -1877,14 +1878,14 @@
       <c r="E76" s="6">
         <v>140900</v>
       </c>
-      <c r="F76" s="9">
+      <c r="F76" s="11">
         <v>3063.04</v>
       </c>
-      <c r="G76" s="9"/>
+      <c r="G76" s="11"/>
     </row>
     <row r="77" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="10"/>
-      <c r="B77" s="10"/>
+      <c r="A77" s="12"/>
+      <c r="B77" s="12"/>
       <c r="C77" s="1" t="s">
         <v>18</v>
       </c>
@@ -1894,14 +1895,14 @@
       <c r="E77" s="6">
         <v>102960</v>
       </c>
-      <c r="F77" s="9">
+      <c r="F77" s="11">
         <v>2782.7</v>
       </c>
-      <c r="G77" s="9"/>
+      <c r="G77" s="11"/>
     </row>
     <row r="78" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10"/>
-      <c r="B78" s="10"/>
+      <c r="A78" s="12"/>
+      <c r="B78" s="12"/>
       <c r="C78" s="1" t="s">
         <v>19</v>
       </c>
@@ -1911,14 +1912,14 @@
       <c r="E78" s="6">
         <v>136800</v>
       </c>
-      <c r="F78" s="9">
+      <c r="F78" s="11">
         <v>2910.64</v>
       </c>
-      <c r="G78" s="9"/>
+      <c r="G78" s="11"/>
     </row>
     <row r="79" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="10"/>
-      <c r="B79" s="10"/>
+      <c r="A79" s="12"/>
+      <c r="B79" s="12"/>
       <c r="C79" s="1" t="s">
         <v>20</v>
       </c>
@@ -1928,14 +1929,14 @@
       <c r="E79" s="6">
         <v>176510</v>
       </c>
-      <c r="F79" s="9">
+      <c r="F79" s="11">
         <v>3460.98</v>
       </c>
-      <c r="G79" s="9"/>
+      <c r="G79" s="11"/>
     </row>
     <row r="80" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10"/>
-      <c r="B80" s="10"/>
+      <c r="A80" s="12"/>
+      <c r="B80" s="12"/>
       <c r="C80" s="1" t="s">
         <v>21</v>
       </c>
@@ -1945,14 +1946,14 @@
       <c r="E80" s="6">
         <v>222360</v>
       </c>
-      <c r="F80" s="9">
+      <c r="F80" s="11">
         <v>3706</v>
       </c>
-      <c r="G80" s="9"/>
+      <c r="G80" s="11"/>
     </row>
     <row r="81" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10"/>
-      <c r="B81" s="10"/>
+      <c r="A81" s="12"/>
+      <c r="B81" s="12"/>
       <c r="C81" s="1" t="s">
         <v>22</v>
       </c>
@@ -1962,14 +1963,14 @@
       <c r="E81" s="6">
         <v>264650</v>
       </c>
-      <c r="F81" s="9">
+      <c r="F81" s="11">
         <v>4268.55</v>
       </c>
-      <c r="G81" s="9"/>
+      <c r="G81" s="11"/>
     </row>
     <row r="82" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="10"/>
-      <c r="B82" s="10"/>
+      <c r="A82" s="12"/>
+      <c r="B82" s="12"/>
       <c r="C82" s="1" t="s">
         <v>23</v>
       </c>
@@ -1979,14 +1980,14 @@
       <c r="E82" s="6">
         <v>131010</v>
       </c>
-      <c r="F82" s="9">
+      <c r="F82" s="11">
         <v>3540.81</v>
       </c>
-      <c r="G82" s="9"/>
+      <c r="G82" s="11"/>
     </row>
     <row r="83" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="10"/>
-      <c r="B83" s="10"/>
+      <c r="A83" s="12"/>
+      <c r="B83" s="12"/>
       <c r="C83" s="1" t="s">
         <v>24</v>
       </c>
@@ -1996,14 +1997,14 @@
       <c r="E83" s="6">
         <v>60000</v>
       </c>
-      <c r="F83" s="9">
+      <c r="F83" s="11">
         <v>2307.69</v>
       </c>
-      <c r="G83" s="9"/>
+      <c r="G83" s="11"/>
     </row>
     <row r="84" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="10"/>
-      <c r="B84" s="10"/>
+      <c r="A84" s="12"/>
+      <c r="B84" s="12"/>
       <c r="C84" s="1" t="s">
         <v>25</v>
       </c>
@@ -2013,30 +2014,30 @@
       <c r="E84" s="6">
         <v>10750</v>
       </c>
-      <c r="F84" s="9">
+      <c r="F84" s="11">
         <v>2150</v>
       </c>
-      <c r="G84" s="9"/>
+      <c r="G84" s="11"/>
     </row>
     <row r="85" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="10"/>
-      <c r="B85" s="8" t="s">
+      <c r="A85" s="12"/>
+      <c r="B85" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C85" s="8"/>
+      <c r="C85" s="13"/>
       <c r="D85" s="5">
         <v>530</v>
       </c>
       <c r="E85" s="6">
         <v>1748490</v>
       </c>
-      <c r="F85" s="9">
+      <c r="F85" s="11">
         <v>3299.04</v>
       </c>
-      <c r="G85" s="9"/>
+      <c r="G85" s="11"/>
     </row>
     <row r="86" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="10"/>
+      <c r="A86" s="12"/>
       <c r="B86" s="4">
         <v>46284</v>
       </c>
@@ -2049,14 +2050,14 @@
       <c r="E86" s="6">
         <v>10700</v>
       </c>
-      <c r="F86" s="9">
+      <c r="F86" s="11">
         <v>10700</v>
       </c>
-      <c r="G86" s="9"/>
+      <c r="G86" s="11"/>
     </row>
     <row r="87" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="10"/>
-      <c r="B87" s="10"/>
+      <c r="A87" s="12"/>
+      <c r="B87" s="12"/>
       <c r="C87" s="1" t="s">
         <v>12</v>
       </c>
@@ -2066,14 +2067,14 @@
       <c r="E87" s="6">
         <v>20600</v>
       </c>
-      <c r="F87" s="9">
+      <c r="F87" s="11">
         <v>3433.33</v>
       </c>
-      <c r="G87" s="9"/>
+      <c r="G87" s="11"/>
     </row>
     <row r="88" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="10"/>
-      <c r="B88" s="10"/>
+      <c r="A88" s="12"/>
+      <c r="B88" s="12"/>
       <c r="C88" s="1" t="s">
         <v>13</v>
       </c>
@@ -2083,14 +2084,14 @@
       <c r="E88" s="6">
         <v>45550</v>
       </c>
-      <c r="F88" s="9">
+      <c r="F88" s="11">
         <v>3253.57</v>
       </c>
-      <c r="G88" s="9"/>
+      <c r="G88" s="11"/>
     </row>
     <row r="89" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="10"/>
-      <c r="B89" s="10"/>
+      <c r="A89" s="12"/>
+      <c r="B89" s="12"/>
       <c r="C89" s="1" t="s">
         <v>14</v>
       </c>
@@ -2100,14 +2101,14 @@
       <c r="E89" s="6">
         <v>129800</v>
       </c>
-      <c r="F89" s="9">
+      <c r="F89" s="11">
         <v>4187.1000000000004</v>
       </c>
-      <c r="G89" s="9"/>
+      <c r="G89" s="11"/>
     </row>
     <row r="90" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="10"/>
-      <c r="B90" s="10"/>
+      <c r="A90" s="12"/>
+      <c r="B90" s="12"/>
       <c r="C90" s="1" t="s">
         <v>15</v>
       </c>
@@ -2117,14 +2118,14 @@
       <c r="E90" s="6">
         <v>179750</v>
       </c>
-      <c r="F90" s="9">
+      <c r="F90" s="11">
         <v>3456.73</v>
       </c>
-      <c r="G90" s="9"/>
+      <c r="G90" s="11"/>
     </row>
     <row r="91" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="10"/>
-      <c r="B91" s="10"/>
+      <c r="A91" s="12"/>
+      <c r="B91" s="12"/>
       <c r="C91" s="1" t="s">
         <v>16</v>
       </c>
@@ -2134,14 +2135,14 @@
       <c r="E91" s="6">
         <v>218860</v>
       </c>
-      <c r="F91" s="9">
+      <c r="F91" s="11">
         <v>3218.53</v>
       </c>
-      <c r="G91" s="9"/>
+      <c r="G91" s="11"/>
     </row>
     <row r="92" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="10"/>
-      <c r="B92" s="10"/>
+      <c r="A92" s="12"/>
+      <c r="B92" s="12"/>
       <c r="C92" s="1" t="s">
         <v>17</v>
       </c>
@@ -2151,14 +2152,14 @@
       <c r="E92" s="6">
         <v>245160</v>
       </c>
-      <c r="F92" s="9">
+      <c r="F92" s="11">
         <v>3183.9</v>
       </c>
-      <c r="G92" s="9"/>
+      <c r="G92" s="11"/>
     </row>
     <row r="93" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="10"/>
-      <c r="B93" s="10"/>
+      <c r="A93" s="12"/>
+      <c r="B93" s="12"/>
       <c r="C93" s="1" t="s">
         <v>18</v>
       </c>
@@ -2168,14 +2169,14 @@
       <c r="E93" s="6">
         <v>316920</v>
       </c>
-      <c r="F93" s="9">
+      <c r="F93" s="11">
         <v>4011.65</v>
       </c>
-      <c r="G93" s="9"/>
+      <c r="G93" s="11"/>
     </row>
     <row r="94" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="10"/>
-      <c r="B94" s="10"/>
+      <c r="A94" s="12"/>
+      <c r="B94" s="12"/>
       <c r="C94" s="1" t="s">
         <v>19</v>
       </c>
@@ -2185,14 +2186,14 @@
       <c r="E94" s="6">
         <v>300250</v>
       </c>
-      <c r="F94" s="9">
+      <c r="F94" s="11">
         <v>3661.59</v>
       </c>
-      <c r="G94" s="9"/>
+      <c r="G94" s="11"/>
     </row>
     <row r="95" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="10"/>
-      <c r="B95" s="10"/>
+      <c r="A95" s="12"/>
+      <c r="B95" s="12"/>
       <c r="C95" s="1" t="s">
         <v>20</v>
       </c>
@@ -2202,14 +2203,14 @@
       <c r="E95" s="6">
         <v>296760</v>
       </c>
-      <c r="F95" s="9">
+      <c r="F95" s="11">
         <v>3532.86</v>
       </c>
-      <c r="G95" s="9"/>
+      <c r="G95" s="11"/>
     </row>
     <row r="96" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="10"/>
-      <c r="B96" s="10"/>
+      <c r="A96" s="12"/>
+      <c r="B96" s="12"/>
       <c r="C96" s="1" t="s">
         <v>21</v>
       </c>
@@ -2219,14 +2220,14 @@
       <c r="E96" s="6">
         <v>289690</v>
       </c>
-      <c r="F96" s="9">
+      <c r="F96" s="11">
         <v>3448.69</v>
       </c>
-      <c r="G96" s="9"/>
+      <c r="G96" s="11"/>
     </row>
     <row r="97" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="10"/>
-      <c r="B97" s="10"/>
+      <c r="A97" s="12"/>
+      <c r="B97" s="12"/>
       <c r="C97" s="1" t="s">
         <v>22</v>
       </c>
@@ -2236,14 +2237,14 @@
       <c r="E97" s="6">
         <v>217960</v>
       </c>
-      <c r="F97" s="9">
+      <c r="F97" s="11">
         <v>3027.22</v>
       </c>
-      <c r="G97" s="9"/>
+      <c r="G97" s="11"/>
     </row>
     <row r="98" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="10"/>
-      <c r="B98" s="10"/>
+      <c r="A98" s="12"/>
+      <c r="B98" s="12"/>
       <c r="C98" s="1" t="s">
         <v>23</v>
       </c>
@@ -2253,14 +2254,14 @@
       <c r="E98" s="6">
         <v>177360</v>
       </c>
-      <c r="F98" s="9">
+      <c r="F98" s="11">
         <v>3224.73</v>
       </c>
-      <c r="G98" s="9"/>
+      <c r="G98" s="11"/>
     </row>
     <row r="99" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="10"/>
-      <c r="B99" s="10"/>
+      <c r="A99" s="12"/>
+      <c r="B99" s="12"/>
       <c r="C99" s="1" t="s">
         <v>24</v>
       </c>
@@ -2270,14 +2271,14 @@
       <c r="E99" s="6">
         <v>78350</v>
       </c>
-      <c r="F99" s="9">
+      <c r="F99" s="11">
         <v>3264.58</v>
       </c>
-      <c r="G99" s="9"/>
+      <c r="G99" s="11"/>
     </row>
     <row r="100" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="10"/>
-      <c r="B100" s="10"/>
+      <c r="A100" s="12"/>
+      <c r="B100" s="12"/>
       <c r="C100" s="1" t="s">
         <v>25</v>
       </c>
@@ -2287,30 +2288,30 @@
       <c r="E100" s="6">
         <v>31650</v>
       </c>
-      <c r="F100" s="9">
+      <c r="F100" s="11">
         <v>4521.43</v>
       </c>
-      <c r="G100" s="9"/>
+      <c r="G100" s="11"/>
     </row>
     <row r="101" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="10"/>
-      <c r="B101" s="8" t="s">
+      <c r="A101" s="12"/>
+      <c r="B101" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C101" s="8"/>
+      <c r="C101" s="13"/>
       <c r="D101" s="5">
         <v>736</v>
       </c>
       <c r="E101" s="6">
         <v>2559360</v>
       </c>
-      <c r="F101" s="9">
+      <c r="F101" s="11">
         <v>3477.39</v>
       </c>
-      <c r="G101" s="9"/>
+      <c r="G101" s="11"/>
     </row>
     <row r="102" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="10"/>
+      <c r="A102" s="12"/>
       <c r="B102" s="4">
         <v>46285</v>
       </c>
@@ -2323,14 +2324,14 @@
       <c r="E102" s="6">
         <v>6100</v>
       </c>
-      <c r="F102" s="9">
+      <c r="F102" s="11">
         <v>2033.33</v>
       </c>
-      <c r="G102" s="9"/>
+      <c r="G102" s="11"/>
     </row>
     <row r="103" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="10"/>
-      <c r="B103" s="10"/>
+      <c r="A103" s="12"/>
+      <c r="B103" s="12"/>
       <c r="C103" s="1" t="s">
         <v>12</v>
       </c>
@@ -2340,14 +2341,14 @@
       <c r="E103" s="6">
         <v>55550</v>
       </c>
-      <c r="F103" s="9">
+      <c r="F103" s="11">
         <v>7935.71</v>
       </c>
-      <c r="G103" s="9"/>
+      <c r="G103" s="11"/>
     </row>
     <row r="104" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="10"/>
-      <c r="B104" s="10"/>
+      <c r="A104" s="12"/>
+      <c r="B104" s="12"/>
       <c r="C104" s="1" t="s">
         <v>13</v>
       </c>
@@ -2357,14 +2358,14 @@
       <c r="E104" s="6">
         <v>65350</v>
       </c>
-      <c r="F104" s="9">
+      <c r="F104" s="11">
         <v>3844.12</v>
       </c>
-      <c r="G104" s="9"/>
+      <c r="G104" s="11"/>
     </row>
     <row r="105" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="10"/>
-      <c r="B105" s="10"/>
+      <c r="A105" s="12"/>
+      <c r="B105" s="12"/>
       <c r="C105" s="1" t="s">
         <v>14</v>
       </c>
@@ -2374,14 +2375,14 @@
       <c r="E105" s="6">
         <v>105650</v>
       </c>
-      <c r="F105" s="9">
+      <c r="F105" s="11">
         <v>3912.96</v>
       </c>
-      <c r="G105" s="9"/>
+      <c r="G105" s="11"/>
     </row>
     <row r="106" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="10"/>
-      <c r="B106" s="10"/>
+      <c r="A106" s="12"/>
+      <c r="B106" s="12"/>
       <c r="C106" s="1" t="s">
         <v>15</v>
       </c>
@@ -2391,14 +2392,14 @@
       <c r="E106" s="6">
         <v>200400</v>
       </c>
-      <c r="F106" s="9">
+      <c r="F106" s="11">
         <v>3853.85</v>
       </c>
-      <c r="G106" s="9"/>
+      <c r="G106" s="11"/>
     </row>
     <row r="107" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="10"/>
-      <c r="B107" s="10"/>
+      <c r="A107" s="12"/>
+      <c r="B107" s="12"/>
       <c r="C107" s="1" t="s">
         <v>16</v>
       </c>
@@ -2408,14 +2409,14 @@
       <c r="E107" s="6">
         <v>209300</v>
       </c>
-      <c r="F107" s="9">
+      <c r="F107" s="11">
         <v>3608.62</v>
       </c>
-      <c r="G107" s="9"/>
+      <c r="G107" s="11"/>
     </row>
     <row r="108" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="10"/>
-      <c r="B108" s="10"/>
+      <c r="A108" s="12"/>
+      <c r="B108" s="12"/>
       <c r="C108" s="1" t="s">
         <v>17</v>
       </c>
@@ -2425,14 +2426,14 @@
       <c r="E108" s="6">
         <v>305600</v>
       </c>
-      <c r="F108" s="9">
+      <c r="F108" s="11">
         <v>3772.84</v>
       </c>
-      <c r="G108" s="9"/>
+      <c r="G108" s="11"/>
     </row>
     <row r="109" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="10"/>
-      <c r="B109" s="10"/>
+      <c r="A109" s="12"/>
+      <c r="B109" s="12"/>
       <c r="C109" s="1" t="s">
         <v>18</v>
       </c>
@@ -2442,14 +2443,14 @@
       <c r="E109" s="6">
         <v>280250</v>
       </c>
-      <c r="F109" s="9">
+      <c r="F109" s="11">
         <v>3592.95</v>
       </c>
-      <c r="G109" s="9"/>
+      <c r="G109" s="11"/>
     </row>
     <row r="110" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="10"/>
-      <c r="B110" s="10"/>
+      <c r="A110" s="12"/>
+      <c r="B110" s="12"/>
       <c r="C110" s="1" t="s">
         <v>19</v>
       </c>
@@ -2459,14 +2460,14 @@
       <c r="E110" s="6">
         <v>202510</v>
       </c>
-      <c r="F110" s="9">
+      <c r="F110" s="11">
         <v>3616.25</v>
       </c>
-      <c r="G110" s="9"/>
+      <c r="G110" s="11"/>
     </row>
     <row r="111" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A111" s="10"/>
-      <c r="B111" s="10"/>
+      <c r="A111" s="12"/>
+      <c r="B111" s="12"/>
       <c r="C111" s="1" t="s">
         <v>20</v>
       </c>
@@ -2476,14 +2477,14 @@
       <c r="E111" s="6">
         <v>205010</v>
       </c>
-      <c r="F111" s="9">
+      <c r="F111" s="11">
         <v>3360.82</v>
       </c>
-      <c r="G111" s="9"/>
+      <c r="G111" s="11"/>
     </row>
     <row r="112" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="10"/>
-      <c r="B112" s="10"/>
+      <c r="A112" s="12"/>
+      <c r="B112" s="12"/>
       <c r="C112" s="1" t="s">
         <v>21</v>
       </c>
@@ -2493,14 +2494,14 @@
       <c r="E112" s="6">
         <v>199350</v>
       </c>
-      <c r="F112" s="9">
+      <c r="F112" s="11">
         <v>3497.37</v>
       </c>
-      <c r="G112" s="9"/>
+      <c r="G112" s="11"/>
     </row>
     <row r="113" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="10"/>
-      <c r="B113" s="10"/>
+      <c r="A113" s="12"/>
+      <c r="B113" s="12"/>
       <c r="C113" s="1" t="s">
         <v>22</v>
       </c>
@@ -2510,14 +2511,14 @@
       <c r="E113" s="6">
         <v>213900</v>
       </c>
-      <c r="F113" s="9">
+      <c r="F113" s="11">
         <v>3506.56</v>
       </c>
-      <c r="G113" s="9"/>
+      <c r="G113" s="11"/>
     </row>
     <row r="114" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="10"/>
-      <c r="B114" s="10"/>
+      <c r="A114" s="12"/>
+      <c r="B114" s="12"/>
       <c r="C114" s="1" t="s">
         <v>23</v>
       </c>
@@ -2527,14 +2528,14 @@
       <c r="E114" s="6">
         <v>132960</v>
       </c>
-      <c r="F114" s="9">
+      <c r="F114" s="11">
         <v>3693.33</v>
       </c>
-      <c r="G114" s="9"/>
+      <c r="G114" s="11"/>
     </row>
     <row r="115" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="10"/>
-      <c r="B115" s="10"/>
+      <c r="A115" s="12"/>
+      <c r="B115" s="12"/>
       <c r="C115" s="1" t="s">
         <v>24</v>
       </c>
@@ -2544,14 +2545,14 @@
       <c r="E115" s="6">
         <v>31300</v>
       </c>
-      <c r="F115" s="9">
+      <c r="F115" s="11">
         <v>2407.69</v>
       </c>
-      <c r="G115" s="9"/>
+      <c r="G115" s="11"/>
     </row>
     <row r="116" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="10"/>
-      <c r="B116" s="10"/>
+      <c r="A116" s="12"/>
+      <c r="B116" s="12"/>
       <c r="C116" s="1" t="s">
         <v>25</v>
       </c>
@@ -2561,30 +2562,30 @@
       <c r="E116" s="6">
         <v>30670</v>
       </c>
-      <c r="F116" s="9">
+      <c r="F116" s="11">
         <v>3067</v>
       </c>
-      <c r="G116" s="9"/>
+      <c r="G116" s="11"/>
     </row>
     <row r="117" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A117" s="10"/>
-      <c r="B117" s="8" t="s">
+      <c r="A117" s="12"/>
+      <c r="B117" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C117" s="8"/>
+      <c r="C117" s="13"/>
       <c r="D117" s="5">
         <v>617</v>
       </c>
       <c r="E117" s="6">
         <v>2243900</v>
       </c>
-      <c r="F117" s="9">
+      <c r="F117" s="11">
         <v>3636.79</v>
       </c>
-      <c r="G117" s="9"/>
+      <c r="G117" s="11"/>
     </row>
     <row r="118" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="10"/>
+      <c r="A118" s="12"/>
       <c r="B118" s="4">
         <v>46286</v>
       </c>
@@ -2597,14 +2598,14 @@
       <c r="E118" s="6">
         <v>5050</v>
       </c>
-      <c r="F118" s="9">
+      <c r="F118" s="11">
         <v>1683.33</v>
       </c>
-      <c r="G118" s="9"/>
+      <c r="G118" s="11"/>
     </row>
     <row r="119" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="10"/>
-      <c r="B119" s="10"/>
+      <c r="A119" s="12"/>
+      <c r="B119" s="12"/>
       <c r="C119" s="1" t="s">
         <v>13</v>
       </c>
@@ -2614,14 +2615,14 @@
       <c r="E119" s="6">
         <v>37050</v>
       </c>
-      <c r="F119" s="9">
+      <c r="F119" s="11">
         <v>2646.43</v>
       </c>
-      <c r="G119" s="9"/>
+      <c r="G119" s="11"/>
     </row>
     <row r="120" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="10"/>
-      <c r="B120" s="10"/>
+      <c r="A120" s="12"/>
+      <c r="B120" s="12"/>
       <c r="C120" s="1" t="s">
         <v>14</v>
       </c>
@@ -2631,14 +2632,14 @@
       <c r="E120" s="6">
         <v>91700</v>
       </c>
-      <c r="F120" s="9">
+      <c r="F120" s="11">
         <v>2865.63</v>
       </c>
-      <c r="G120" s="9"/>
+      <c r="G120" s="11"/>
     </row>
     <row r="121" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="10"/>
-      <c r="B121" s="10"/>
+      <c r="A121" s="12"/>
+      <c r="B121" s="12"/>
       <c r="C121" s="1" t="s">
         <v>15</v>
       </c>
@@ -2648,14 +2649,14 @@
       <c r="E121" s="6">
         <v>203250</v>
       </c>
-      <c r="F121" s="9">
+      <c r="F121" s="11">
         <v>4418.4799999999996</v>
       </c>
-      <c r="G121" s="9"/>
+      <c r="G121" s="11"/>
     </row>
     <row r="122" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="10"/>
-      <c r="B122" s="10"/>
+      <c r="A122" s="12"/>
+      <c r="B122" s="12"/>
       <c r="C122" s="1" t="s">
         <v>16</v>
       </c>
@@ -2665,14 +2666,14 @@
       <c r="E122" s="6">
         <v>125010</v>
       </c>
-      <c r="F122" s="9">
+      <c r="F122" s="11">
         <v>3205.38</v>
       </c>
-      <c r="G122" s="9"/>
+      <c r="G122" s="11"/>
     </row>
     <row r="123" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="10"/>
-      <c r="B123" s="10"/>
+      <c r="A123" s="12"/>
+      <c r="B123" s="12"/>
       <c r="C123" s="1" t="s">
         <v>17</v>
       </c>
@@ -2682,14 +2683,14 @@
       <c r="E123" s="6">
         <v>103100</v>
       </c>
-      <c r="F123" s="9">
+      <c r="F123" s="11">
         <v>3032.35</v>
       </c>
-      <c r="G123" s="9"/>
+      <c r="G123" s="11"/>
     </row>
     <row r="124" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="10"/>
-      <c r="B124" s="10"/>
+      <c r="A124" s="12"/>
+      <c r="B124" s="12"/>
       <c r="C124" s="1" t="s">
         <v>18</v>
       </c>
@@ -2699,14 +2700,14 @@
       <c r="E124" s="6">
         <v>118360</v>
       </c>
-      <c r="F124" s="9">
+      <c r="F124" s="11">
         <v>2886.83</v>
       </c>
-      <c r="G124" s="9"/>
+      <c r="G124" s="11"/>
     </row>
     <row r="125" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="10"/>
-      <c r="B125" s="10"/>
+      <c r="A125" s="12"/>
+      <c r="B125" s="12"/>
       <c r="C125" s="1" t="s">
         <v>19</v>
       </c>
@@ -2716,14 +2717,14 @@
       <c r="E125" s="6">
         <v>92270</v>
       </c>
-      <c r="F125" s="9">
+      <c r="F125" s="11">
         <v>2563.06</v>
       </c>
-      <c r="G125" s="9"/>
+      <c r="G125" s="11"/>
     </row>
     <row r="126" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="10"/>
-      <c r="B126" s="10"/>
+      <c r="A126" s="12"/>
+      <c r="B126" s="12"/>
       <c r="C126" s="1" t="s">
         <v>20</v>
       </c>
@@ -2733,14 +2734,14 @@
       <c r="E126" s="6">
         <v>76810</v>
       </c>
-      <c r="F126" s="9">
+      <c r="F126" s="11">
         <v>2743.21</v>
       </c>
-      <c r="G126" s="9"/>
+      <c r="G126" s="11"/>
     </row>
     <row r="127" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="10"/>
-      <c r="B127" s="10"/>
+      <c r="A127" s="12"/>
+      <c r="B127" s="12"/>
       <c r="C127" s="1" t="s">
         <v>21</v>
       </c>
@@ -2750,14 +2751,14 @@
       <c r="E127" s="6">
         <v>132520</v>
       </c>
-      <c r="F127" s="9">
+      <c r="F127" s="11">
         <v>3081.86</v>
       </c>
-      <c r="G127" s="9"/>
+      <c r="G127" s="11"/>
     </row>
     <row r="128" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="10"/>
-      <c r="B128" s="10"/>
+      <c r="A128" s="12"/>
+      <c r="B128" s="12"/>
       <c r="C128" s="1" t="s">
         <v>22</v>
       </c>
@@ -2767,14 +2768,14 @@
       <c r="E128" s="6">
         <v>73560</v>
       </c>
-      <c r="F128" s="9">
+      <c r="F128" s="11">
         <v>3065</v>
       </c>
-      <c r="G128" s="9"/>
+      <c r="G128" s="11"/>
     </row>
     <row r="129" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="10"/>
-      <c r="B129" s="10"/>
+      <c r="A129" s="12"/>
+      <c r="B129" s="12"/>
       <c r="C129" s="1" t="s">
         <v>23</v>
       </c>
@@ -2784,14 +2785,14 @@
       <c r="E129" s="6">
         <v>53600</v>
       </c>
-      <c r="F129" s="9">
+      <c r="F129" s="11">
         <v>2552.38</v>
       </c>
-      <c r="G129" s="9"/>
+      <c r="G129" s="11"/>
     </row>
     <row r="130" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="10"/>
-      <c r="B130" s="10"/>
+      <c r="A130" s="12"/>
+      <c r="B130" s="12"/>
       <c r="C130" s="1" t="s">
         <v>24</v>
       </c>
@@ -2801,14 +2802,14 @@
       <c r="E130" s="6">
         <v>25050</v>
       </c>
-      <c r="F130" s="9">
+      <c r="F130" s="11">
         <v>3578.57</v>
       </c>
-      <c r="G130" s="9"/>
+      <c r="G130" s="11"/>
     </row>
     <row r="131" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="10"/>
-      <c r="B131" s="10"/>
+      <c r="A131" s="12"/>
+      <c r="B131" s="12"/>
       <c r="C131" s="1" t="s">
         <v>25</v>
       </c>
@@ -2818,30 +2819,30 @@
       <c r="E131" s="6">
         <v>12750</v>
       </c>
-      <c r="F131" s="9">
+      <c r="F131" s="11">
         <v>4250</v>
       </c>
-      <c r="G131" s="9"/>
+      <c r="G131" s="11"/>
     </row>
     <row r="132" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="10"/>
-      <c r="B132" s="8" t="s">
+      <c r="A132" s="12"/>
+      <c r="B132" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C132" s="8"/>
+      <c r="C132" s="13"/>
       <c r="D132" s="5">
         <v>371</v>
       </c>
       <c r="E132" s="6">
         <v>1150080</v>
       </c>
-      <c r="F132" s="9">
+      <c r="F132" s="11">
         <v>3099.95</v>
       </c>
-      <c r="G132" s="9"/>
+      <c r="G132" s="11"/>
     </row>
     <row r="133" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="10"/>
+      <c r="A133" s="12"/>
       <c r="B133" s="4">
         <v>46287</v>
       </c>
@@ -2854,14 +2855,14 @@
       <c r="E133" s="6">
         <v>3300</v>
       </c>
-      <c r="F133" s="9">
+      <c r="F133" s="11">
         <v>3300</v>
       </c>
-      <c r="G133" s="9"/>
+      <c r="G133" s="11"/>
     </row>
     <row r="134" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="10"/>
-      <c r="B134" s="10"/>
+      <c r="A134" s="12"/>
+      <c r="B134" s="12"/>
       <c r="C134" s="1" t="s">
         <v>12</v>
       </c>
@@ -2871,14 +2872,14 @@
       <c r="E134" s="6">
         <v>28150</v>
       </c>
-      <c r="F134" s="9">
+      <c r="F134" s="11">
         <v>3127.78</v>
       </c>
-      <c r="G134" s="9"/>
+      <c r="G134" s="11"/>
     </row>
     <row r="135" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="10"/>
-      <c r="B135" s="10"/>
+      <c r="A135" s="12"/>
+      <c r="B135" s="12"/>
       <c r="C135" s="1" t="s">
         <v>13</v>
       </c>
@@ -2888,14 +2889,14 @@
       <c r="E135" s="6">
         <v>13910</v>
       </c>
-      <c r="F135" s="9">
+      <c r="F135" s="11">
         <v>1738.75</v>
       </c>
-      <c r="G135" s="9"/>
+      <c r="G135" s="11"/>
     </row>
     <row r="136" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="10"/>
-      <c r="B136" s="10"/>
+      <c r="A136" s="12"/>
+      <c r="B136" s="12"/>
       <c r="C136" s="1" t="s">
         <v>14</v>
       </c>
@@ -2905,14 +2906,14 @@
       <c r="E136" s="6">
         <v>76100</v>
       </c>
-      <c r="F136" s="9">
+      <c r="F136" s="11">
         <v>2818.52</v>
       </c>
-      <c r="G136" s="9"/>
+      <c r="G136" s="11"/>
     </row>
     <row r="137" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="10"/>
-      <c r="B137" s="10"/>
+      <c r="A137" s="12"/>
+      <c r="B137" s="12"/>
       <c r="C137" s="1" t="s">
         <v>15</v>
       </c>
@@ -2922,14 +2923,14 @@
       <c r="E137" s="6">
         <v>125150</v>
       </c>
-      <c r="F137" s="9">
+      <c r="F137" s="11">
         <v>3680.88</v>
       </c>
-      <c r="G137" s="9"/>
+      <c r="G137" s="11"/>
     </row>
     <row r="138" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="10"/>
-      <c r="B138" s="10"/>
+      <c r="A138" s="12"/>
+      <c r="B138" s="12"/>
       <c r="C138" s="1" t="s">
         <v>16</v>
       </c>
@@ -2939,14 +2940,14 @@
       <c r="E138" s="6">
         <v>43250</v>
       </c>
-      <c r="F138" s="9">
+      <c r="F138" s="11">
         <v>2162.5</v>
       </c>
-      <c r="G138" s="9"/>
+      <c r="G138" s="11"/>
     </row>
     <row r="139" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="10"/>
-      <c r="B139" s="10"/>
+      <c r="A139" s="12"/>
+      <c r="B139" s="12"/>
       <c r="C139" s="1" t="s">
         <v>17</v>
       </c>
@@ -2956,14 +2957,14 @@
       <c r="E139" s="6">
         <v>76430</v>
       </c>
-      <c r="F139" s="9">
+      <c r="F139" s="11">
         <v>2388.44</v>
       </c>
-      <c r="G139" s="9"/>
+      <c r="G139" s="11"/>
     </row>
     <row r="140" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="10"/>
-      <c r="B140" s="10"/>
+      <c r="A140" s="12"/>
+      <c r="B140" s="12"/>
       <c r="C140" s="1" t="s">
         <v>18</v>
       </c>
@@ -2973,14 +2974,14 @@
       <c r="E140" s="6">
         <v>143110</v>
       </c>
-      <c r="F140" s="9">
+      <c r="F140" s="11">
         <v>3111.09</v>
       </c>
-      <c r="G140" s="9"/>
+      <c r="G140" s="11"/>
     </row>
     <row r="141" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="10"/>
-      <c r="B141" s="10"/>
+      <c r="A141" s="12"/>
+      <c r="B141" s="12"/>
       <c r="C141" s="1" t="s">
         <v>19</v>
       </c>
@@ -2990,14 +2991,14 @@
       <c r="E141" s="6">
         <v>55300</v>
       </c>
-      <c r="F141" s="9">
+      <c r="F141" s="11">
         <v>2910.53</v>
       </c>
-      <c r="G141" s="9"/>
+      <c r="G141" s="11"/>
     </row>
     <row r="142" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="10"/>
-      <c r="B142" s="10"/>
+      <c r="A142" s="12"/>
+      <c r="B142" s="12"/>
       <c r="C142" s="1" t="s">
         <v>20</v>
       </c>
@@ -3007,14 +3008,14 @@
       <c r="E142" s="6">
         <v>83200</v>
       </c>
-      <c r="F142" s="9">
+      <c r="F142" s="11">
         <v>3328</v>
       </c>
-      <c r="G142" s="9"/>
+      <c r="G142" s="11"/>
     </row>
     <row r="143" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="10"/>
-      <c r="B143" s="10"/>
+      <c r="A143" s="12"/>
+      <c r="B143" s="12"/>
       <c r="C143" s="1" t="s">
         <v>21</v>
       </c>
@@ -3024,14 +3025,14 @@
       <c r="E143" s="6">
         <v>154710</v>
       </c>
-      <c r="F143" s="9">
+      <c r="F143" s="11">
         <v>2762.68</v>
       </c>
-      <c r="G143" s="9"/>
+      <c r="G143" s="11"/>
     </row>
     <row r="144" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="10"/>
-      <c r="B144" s="10"/>
+      <c r="A144" s="12"/>
+      <c r="B144" s="12"/>
       <c r="C144" s="1" t="s">
         <v>22</v>
       </c>
@@ -3041,14 +3042,14 @@
       <c r="E144" s="6">
         <v>46520</v>
       </c>
-      <c r="F144" s="9">
+      <c r="F144" s="11">
         <v>2584.44</v>
       </c>
-      <c r="G144" s="9"/>
+      <c r="G144" s="11"/>
     </row>
     <row r="145" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="10"/>
-      <c r="B145" s="10"/>
+      <c r="A145" s="12"/>
+      <c r="B145" s="12"/>
       <c r="C145" s="1" t="s">
         <v>23</v>
       </c>
@@ -3058,14 +3059,14 @@
       <c r="E145" s="6">
         <v>51200</v>
       </c>
-      <c r="F145" s="9">
+      <c r="F145" s="11">
         <v>2560</v>
       </c>
-      <c r="G145" s="9"/>
+      <c r="G145" s="11"/>
     </row>
     <row r="146" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="10"/>
-      <c r="B146" s="10"/>
+      <c r="A146" s="12"/>
+      <c r="B146" s="12"/>
       <c r="C146" s="1" t="s">
         <v>24</v>
       </c>
@@ -3075,14 +3076,14 @@
       <c r="E146" s="6">
         <v>28480</v>
       </c>
-      <c r="F146" s="9">
+      <c r="F146" s="11">
         <v>2190.77</v>
       </c>
-      <c r="G146" s="9"/>
+      <c r="G146" s="11"/>
     </row>
     <row r="147" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="10"/>
-      <c r="B147" s="10"/>
+      <c r="A147" s="12"/>
+      <c r="B147" s="12"/>
       <c r="C147" s="1" t="s">
         <v>25</v>
       </c>
@@ -3092,30 +3093,30 @@
       <c r="E147" s="6">
         <v>3050</v>
       </c>
-      <c r="F147" s="9">
+      <c r="F147" s="11">
         <v>1525</v>
       </c>
-      <c r="G147" s="9"/>
+      <c r="G147" s="11"/>
     </row>
     <row r="148" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="10"/>
-      <c r="B148" s="8" t="s">
+      <c r="A148" s="12"/>
+      <c r="B148" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C148" s="8"/>
+      <c r="C148" s="13"/>
       <c r="D148" s="5">
         <v>330</v>
       </c>
       <c r="E148" s="6">
         <v>931860</v>
       </c>
-      <c r="F148" s="9">
+      <c r="F148" s="11">
         <v>2823.82</v>
       </c>
-      <c r="G148" s="9"/>
+      <c r="G148" s="11"/>
     </row>
     <row r="149" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="10"/>
+      <c r="A149" s="12"/>
       <c r="B149" s="4">
         <v>46288</v>
       </c>
@@ -3128,14 +3129,14 @@
       <c r="E149" s="6">
         <v>8950</v>
       </c>
-      <c r="F149" s="9">
+      <c r="F149" s="11">
         <v>1790</v>
       </c>
-      <c r="G149" s="9"/>
+      <c r="G149" s="11"/>
     </row>
     <row r="150" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="10"/>
-      <c r="B150" s="10"/>
+      <c r="A150" s="12"/>
+      <c r="B150" s="12"/>
       <c r="C150" s="1" t="s">
         <v>13</v>
       </c>
@@ -3145,14 +3146,14 @@
       <c r="E150" s="6">
         <v>13550</v>
       </c>
-      <c r="F150" s="9">
+      <c r="F150" s="11">
         <v>2710</v>
       </c>
-      <c r="G150" s="9"/>
+      <c r="G150" s="11"/>
     </row>
     <row r="151" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="10"/>
-      <c r="B151" s="10"/>
+      <c r="A151" s="12"/>
+      <c r="B151" s="12"/>
       <c r="C151" s="1" t="s">
         <v>14</v>
       </c>
@@ -3162,14 +3163,14 @@
       <c r="E151" s="6">
         <v>81600</v>
       </c>
-      <c r="F151" s="9">
+      <c r="F151" s="11">
         <v>3138.46</v>
       </c>
-      <c r="G151" s="9"/>
+      <c r="G151" s="11"/>
     </row>
     <row r="152" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="10"/>
-      <c r="B152" s="10"/>
+      <c r="A152" s="12"/>
+      <c r="B152" s="12"/>
       <c r="C152" s="1" t="s">
         <v>15</v>
       </c>
@@ -3179,14 +3180,14 @@
       <c r="E152" s="6">
         <v>83220</v>
       </c>
-      <c r="F152" s="9">
+      <c r="F152" s="11">
         <v>2521.8200000000002</v>
       </c>
-      <c r="G152" s="9"/>
+      <c r="G152" s="11"/>
     </row>
     <row r="153" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="10"/>
-      <c r="B153" s="10"/>
+      <c r="A153" s="12"/>
+      <c r="B153" s="12"/>
       <c r="C153" s="1" t="s">
         <v>16</v>
       </c>
@@ -3196,14 +3197,14 @@
       <c r="E153" s="6">
         <v>76970</v>
       </c>
-      <c r="F153" s="9">
+      <c r="F153" s="11">
         <v>2332.42</v>
       </c>
-      <c r="G153" s="9"/>
+      <c r="G153" s="11"/>
     </row>
     <row r="154" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="10"/>
-      <c r="B154" s="10"/>
+      <c r="A154" s="12"/>
+      <c r="B154" s="12"/>
       <c r="C154" s="1" t="s">
         <v>17</v>
       </c>
@@ -3213,14 +3214,14 @@
       <c r="E154" s="6">
         <v>68300</v>
       </c>
-      <c r="F154" s="9">
+      <c r="F154" s="11">
         <v>2276.67</v>
       </c>
-      <c r="G154" s="9"/>
+      <c r="G154" s="11"/>
     </row>
     <row r="155" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="10"/>
-      <c r="B155" s="10"/>
+      <c r="A155" s="12"/>
+      <c r="B155" s="12"/>
       <c r="C155" s="1" t="s">
         <v>18</v>
       </c>
@@ -3230,14 +3231,14 @@
       <c r="E155" s="6">
         <v>58800</v>
       </c>
-      <c r="F155" s="9">
+      <c r="F155" s="11">
         <v>2450</v>
       </c>
-      <c r="G155" s="9"/>
+      <c r="G155" s="11"/>
     </row>
     <row r="156" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="10"/>
-      <c r="B156" s="10"/>
+      <c r="A156" s="12"/>
+      <c r="B156" s="12"/>
       <c r="C156" s="1" t="s">
         <v>19</v>
       </c>
@@ -3247,14 +3248,14 @@
       <c r="E156" s="6">
         <v>70950</v>
       </c>
-      <c r="F156" s="9">
+      <c r="F156" s="11">
         <v>2728.85</v>
       </c>
-      <c r="G156" s="9"/>
+      <c r="G156" s="11"/>
     </row>
     <row r="157" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="10"/>
-      <c r="B157" s="10"/>
+      <c r="A157" s="12"/>
+      <c r="B157" s="12"/>
       <c r="C157" s="1" t="s">
         <v>20</v>
       </c>
@@ -3264,14 +3265,14 @@
       <c r="E157" s="6">
         <v>98550</v>
       </c>
-      <c r="F157" s="9">
+      <c r="F157" s="11">
         <v>2986.36</v>
       </c>
-      <c r="G157" s="9"/>
+      <c r="G157" s="11"/>
     </row>
     <row r="158" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="10"/>
-      <c r="B158" s="10"/>
+      <c r="A158" s="12"/>
+      <c r="B158" s="12"/>
       <c r="C158" s="1" t="s">
         <v>25</v>
       </c>
@@ -3281,30 +3282,30 @@
       <c r="E158" s="6">
         <v>560</v>
       </c>
-      <c r="F158" s="9">
+      <c r="F158" s="11">
         <v>560</v>
       </c>
-      <c r="G158" s="9"/>
+      <c r="G158" s="11"/>
     </row>
     <row r="159" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="10"/>
-      <c r="B159" s="8" t="s">
+      <c r="A159" s="12"/>
+      <c r="B159" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C159" s="8"/>
+      <c r="C159" s="13"/>
       <c r="D159" s="5">
         <v>216</v>
       </c>
       <c r="E159" s="6">
         <v>561450</v>
       </c>
-      <c r="F159" s="9">
+      <c r="F159" s="11">
         <v>2599.31</v>
       </c>
-      <c r="G159" s="9"/>
+      <c r="G159" s="11"/>
     </row>
     <row r="160" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="10"/>
+      <c r="A160" s="12"/>
       <c r="B160" s="7">
         <v>46289</v>
       </c>
@@ -3317,13 +3318,13 @@
       <c r="E160" s="6">
         <v>5500</v>
       </c>
-      <c r="F160" s="9">
+      <c r="F160" s="11">
         <v>5500</v>
       </c>
-      <c r="G160" s="9"/>
+      <c r="G160" s="11"/>
     </row>
     <row r="161" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="10"/>
+      <c r="A161" s="12"/>
       <c r="B161" s="4">
         <v>46290</v>
       </c>
@@ -3336,14 +3337,14 @@
       <c r="E161" s="6">
         <v>9910</v>
       </c>
-      <c r="F161" s="9">
+      <c r="F161" s="11">
         <v>1238.75</v>
       </c>
-      <c r="G161" s="9"/>
+      <c r="G161" s="11"/>
     </row>
     <row r="162" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="10"/>
-      <c r="B162" s="10"/>
+      <c r="A162" s="12"/>
+      <c r="B162" s="12"/>
       <c r="C162" s="1" t="s">
         <v>13</v>
       </c>
@@ -3353,14 +3354,14 @@
       <c r="E162" s="6">
         <v>9300</v>
       </c>
-      <c r="F162" s="9">
+      <c r="F162" s="11">
         <v>3100</v>
       </c>
-      <c r="G162" s="9"/>
+      <c r="G162" s="11"/>
     </row>
     <row r="163" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="10"/>
-      <c r="B163" s="10"/>
+      <c r="A163" s="12"/>
+      <c r="B163" s="12"/>
       <c r="C163" s="1" t="s">
         <v>14</v>
       </c>
@@ -3370,14 +3371,14 @@
       <c r="E163" s="6">
         <v>130000</v>
       </c>
-      <c r="F163" s="9">
+      <c r="F163" s="11">
         <v>3714.29</v>
       </c>
-      <c r="G163" s="9"/>
+      <c r="G163" s="11"/>
     </row>
     <row r="164" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="10"/>
-      <c r="B164" s="10"/>
+      <c r="A164" s="12"/>
+      <c r="B164" s="12"/>
       <c r="C164" s="1" t="s">
         <v>15</v>
       </c>
@@ -3387,14 +3388,14 @@
       <c r="E164" s="6">
         <v>228160</v>
       </c>
-      <c r="F164" s="9">
+      <c r="F164" s="11">
         <v>3867.12</v>
       </c>
-      <c r="G164" s="9"/>
+      <c r="G164" s="11"/>
     </row>
     <row r="165" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="10"/>
-      <c r="B165" s="10"/>
+      <c r="A165" s="12"/>
+      <c r="B165" s="12"/>
       <c r="C165" s="1" t="s">
         <v>16</v>
       </c>
@@ -3404,14 +3405,14 @@
       <c r="E165" s="6">
         <v>132870</v>
       </c>
-      <c r="F165" s="9">
+      <c r="F165" s="11">
         <v>3240.73</v>
       </c>
-      <c r="G165" s="9"/>
+      <c r="G165" s="11"/>
     </row>
     <row r="166" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="10"/>
-      <c r="B166" s="10"/>
+      <c r="A166" s="12"/>
+      <c r="B166" s="12"/>
       <c r="C166" s="1" t="s">
         <v>17</v>
       </c>
@@ -3421,14 +3422,14 @@
       <c r="E166" s="6">
         <v>204590</v>
       </c>
-      <c r="F166" s="9">
+      <c r="F166" s="11">
         <v>3099.85</v>
       </c>
-      <c r="G166" s="9"/>
+      <c r="G166" s="11"/>
     </row>
     <row r="167" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="10"/>
-      <c r="B167" s="10"/>
+      <c r="A167" s="12"/>
+      <c r="B167" s="12"/>
       <c r="C167" s="1" t="s">
         <v>18</v>
       </c>
@@ -3438,14 +3439,14 @@
       <c r="E167" s="6">
         <v>122420</v>
       </c>
-      <c r="F167" s="9">
+      <c r="F167" s="11">
         <v>3497.71</v>
       </c>
-      <c r="G167" s="9"/>
+      <c r="G167" s="11"/>
     </row>
     <row r="168" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="10"/>
-      <c r="B168" s="10"/>
+      <c r="A168" s="12"/>
+      <c r="B168" s="12"/>
       <c r="C168" s="1" t="s">
         <v>19</v>
       </c>
@@ -3455,14 +3456,14 @@
       <c r="E168" s="6">
         <v>193140</v>
       </c>
-      <c r="F168" s="9">
+      <c r="F168" s="11">
         <v>3941.63</v>
       </c>
-      <c r="G168" s="9"/>
+      <c r="G168" s="11"/>
     </row>
     <row r="169" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="10"/>
-      <c r="B169" s="10"/>
+      <c r="A169" s="12"/>
+      <c r="B169" s="12"/>
       <c r="C169" s="1" t="s">
         <v>20</v>
       </c>
@@ -3472,14 +3473,14 @@
       <c r="E169" s="6">
         <v>187820</v>
       </c>
-      <c r="F169" s="9">
+      <c r="F169" s="11">
         <v>3183.39</v>
       </c>
-      <c r="G169" s="9"/>
+      <c r="G169" s="11"/>
     </row>
     <row r="170" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="10"/>
-      <c r="B170" s="10"/>
+      <c r="A170" s="12"/>
+      <c r="B170" s="12"/>
       <c r="C170" s="1" t="s">
         <v>21</v>
       </c>
@@ -3489,14 +3490,14 @@
       <c r="E170" s="6">
         <v>397060</v>
       </c>
-      <c r="F170" s="9">
+      <c r="F170" s="11">
         <v>4315.87</v>
       </c>
-      <c r="G170" s="9"/>
+      <c r="G170" s="11"/>
     </row>
     <row r="171" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="10"/>
-      <c r="B171" s="10"/>
+      <c r="A171" s="12"/>
+      <c r="B171" s="12"/>
       <c r="C171" s="1" t="s">
         <v>22</v>
       </c>
@@ -3506,14 +3507,14 @@
       <c r="E171" s="6">
         <v>293020</v>
       </c>
-      <c r="F171" s="9">
+      <c r="F171" s="11">
         <v>4013.97</v>
       </c>
-      <c r="G171" s="9"/>
+      <c r="G171" s="11"/>
     </row>
     <row r="172" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A172" s="10"/>
-      <c r="B172" s="10"/>
+      <c r="A172" s="12"/>
+      <c r="B172" s="12"/>
       <c r="C172" s="1" t="s">
         <v>23</v>
       </c>
@@ -3523,14 +3524,14 @@
       <c r="E172" s="6">
         <v>162250</v>
       </c>
-      <c r="F172" s="9">
+      <c r="F172" s="11">
         <v>3527.17</v>
       </c>
-      <c r="G172" s="9"/>
+      <c r="G172" s="11"/>
     </row>
     <row r="173" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="10"/>
-      <c r="B173" s="10"/>
+      <c r="A173" s="12"/>
+      <c r="B173" s="12"/>
       <c r="C173" s="1" t="s">
         <v>24</v>
       </c>
@@ -3540,14 +3541,14 @@
       <c r="E173" s="6">
         <v>99500</v>
       </c>
-      <c r="F173" s="9">
+      <c r="F173" s="11">
         <v>3431.03</v>
       </c>
-      <c r="G173" s="9"/>
+      <c r="G173" s="11"/>
     </row>
     <row r="174" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A174" s="10"/>
-      <c r="B174" s="10"/>
+      <c r="A174" s="12"/>
+      <c r="B174" s="12"/>
       <c r="C174" s="1" t="s">
         <v>25</v>
       </c>
@@ -3557,17 +3558,17 @@
       <c r="E174" s="6">
         <v>17050</v>
       </c>
-      <c r="F174" s="9">
+      <c r="F174" s="11">
         <v>1420.83</v>
       </c>
-      <c r="G174" s="9"/>
+      <c r="G174" s="11"/>
     </row>
     <row r="175" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A175" s="10"/>
-      <c r="B175" s="8" t="s">
+      <c r="A175" s="12"/>
+      <c r="B175" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C175" s="8"/>
+      <c r="C175" s="13"/>
       <c r="D175" s="5">
         <f>SUM(D174,D161)</f>
         <v>20</v>
@@ -3575,13 +3576,13 @@
       <c r="E175" s="6">
         <v>2187090</v>
       </c>
-      <c r="F175" s="9">
+      <c r="F175" s="11">
         <v>3603.11</v>
       </c>
-      <c r="G175" s="9"/>
+      <c r="G175" s="11"/>
     </row>
     <row r="176" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="10"/>
+      <c r="A176" s="12"/>
       <c r="B176" s="4">
         <v>46291</v>
       </c>
@@ -3594,14 +3595,14 @@
       <c r="E176" s="6">
         <v>13900</v>
       </c>
-      <c r="F176" s="9">
+      <c r="F176" s="11">
         <v>4633.33</v>
       </c>
-      <c r="G176" s="9"/>
+      <c r="G176" s="11"/>
     </row>
     <row r="177" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A177" s="10"/>
-      <c r="B177" s="10"/>
+      <c r="A177" s="12"/>
+      <c r="B177" s="12"/>
       <c r="C177" s="1" t="s">
         <v>13</v>
       </c>
@@ -3611,14 +3612,14 @@
       <c r="E177" s="6">
         <v>34610</v>
       </c>
-      <c r="F177" s="9">
+      <c r="F177" s="11">
         <v>3461</v>
       </c>
-      <c r="G177" s="9"/>
+      <c r="G177" s="11"/>
     </row>
     <row r="178" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A178" s="10"/>
-      <c r="B178" s="10"/>
+      <c r="A178" s="12"/>
+      <c r="B178" s="12"/>
       <c r="C178" s="1" t="s">
         <v>14</v>
       </c>
@@ -3628,14 +3629,14 @@
       <c r="E178" s="6">
         <v>107000</v>
       </c>
-      <c r="F178" s="9">
+      <c r="F178" s="11">
         <v>3821.43</v>
       </c>
-      <c r="G178" s="9"/>
+      <c r="G178" s="11"/>
     </row>
     <row r="179" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A179" s="10"/>
-      <c r="B179" s="10"/>
+      <c r="A179" s="12"/>
+      <c r="B179" s="12"/>
       <c r="C179" s="1" t="s">
         <v>15</v>
       </c>
@@ -3645,14 +3646,14 @@
       <c r="E179" s="6">
         <v>99730</v>
       </c>
-      <c r="F179" s="9">
+      <c r="F179" s="11">
         <v>2933.24</v>
       </c>
-      <c r="G179" s="9"/>
+      <c r="G179" s="11"/>
     </row>
     <row r="180" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A180" s="10"/>
-      <c r="B180" s="10"/>
+      <c r="A180" s="12"/>
+      <c r="B180" s="12"/>
       <c r="C180" s="1" t="s">
         <v>16</v>
       </c>
@@ -3662,14 +3663,14 @@
       <c r="E180" s="6">
         <v>373710</v>
       </c>
-      <c r="F180" s="9">
+      <c r="F180" s="11">
         <v>3774.85</v>
       </c>
-      <c r="G180" s="9"/>
+      <c r="G180" s="11"/>
     </row>
     <row r="181" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A181" s="10"/>
-      <c r="B181" s="10"/>
+      <c r="A181" s="12"/>
+      <c r="B181" s="12"/>
       <c r="C181" s="1" t="s">
         <v>17</v>
       </c>
@@ -3679,14 +3680,14 @@
       <c r="E181" s="6">
         <v>354310</v>
       </c>
-      <c r="F181" s="9">
+      <c r="F181" s="11">
         <v>4787.97</v>
       </c>
-      <c r="G181" s="9"/>
+      <c r="G181" s="11"/>
     </row>
     <row r="182" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A182" s="10"/>
-      <c r="B182" s="10"/>
+      <c r="A182" s="12"/>
+      <c r="B182" s="12"/>
       <c r="C182" s="1" t="s">
         <v>18</v>
       </c>
@@ -3696,14 +3697,14 @@
       <c r="E182" s="6">
         <v>265980</v>
       </c>
-      <c r="F182" s="9">
+      <c r="F182" s="11">
         <v>3283.7</v>
       </c>
-      <c r="G182" s="9"/>
+      <c r="G182" s="11"/>
     </row>
     <row r="183" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A183" s="10"/>
-      <c r="B183" s="10"/>
+      <c r="A183" s="12"/>
+      <c r="B183" s="12"/>
       <c r="C183" s="1" t="s">
         <v>19</v>
       </c>
@@ -3713,14 +3714,14 @@
       <c r="E183" s="6">
         <v>318950</v>
       </c>
-      <c r="F183" s="9">
+      <c r="F183" s="11">
         <v>3752.35</v>
       </c>
-      <c r="G183" s="9"/>
+      <c r="G183" s="11"/>
     </row>
     <row r="184" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="10"/>
-      <c r="B184" s="10"/>
+      <c r="A184" s="12"/>
+      <c r="B184" s="12"/>
       <c r="C184" s="1" t="s">
         <v>20</v>
       </c>
@@ -3730,14 +3731,14 @@
       <c r="E184" s="6">
         <v>283420</v>
       </c>
-      <c r="F184" s="9">
+      <c r="F184" s="11">
         <v>3374.05</v>
       </c>
-      <c r="G184" s="9"/>
+      <c r="G184" s="11"/>
     </row>
     <row r="185" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A185" s="10"/>
-      <c r="B185" s="10"/>
+      <c r="A185" s="12"/>
+      <c r="B185" s="12"/>
       <c r="C185" s="1" t="s">
         <v>21</v>
       </c>
@@ -3747,14 +3748,14 @@
       <c r="E185" s="6">
         <v>399400</v>
       </c>
-      <c r="F185" s="9">
+      <c r="F185" s="11">
         <v>4204.21</v>
       </c>
-      <c r="G185" s="9"/>
+      <c r="G185" s="11"/>
     </row>
     <row r="186" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" s="10"/>
-      <c r="B186" s="10"/>
+      <c r="A186" s="12"/>
+      <c r="B186" s="12"/>
       <c r="C186" s="1" t="s">
         <v>22</v>
       </c>
@@ -3764,14 +3765,14 @@
       <c r="E186" s="6">
         <v>226450</v>
       </c>
-      <c r="F186" s="9">
+      <c r="F186" s="11">
         <v>3060.14</v>
       </c>
-      <c r="G186" s="9"/>
+      <c r="G186" s="11"/>
     </row>
     <row r="187" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A187" s="10"/>
-      <c r="B187" s="10"/>
+      <c r="A187" s="12"/>
+      <c r="B187" s="12"/>
       <c r="C187" s="1" t="s">
         <v>23</v>
       </c>
@@ -3781,14 +3782,14 @@
       <c r="E187" s="6">
         <v>219410</v>
       </c>
-      <c r="F187" s="9">
+      <c r="F187" s="11">
         <v>2384.89</v>
       </c>
-      <c r="G187" s="9"/>
+      <c r="G187" s="11"/>
     </row>
     <row r="188" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A188" s="10"/>
-      <c r="B188" s="10"/>
+      <c r="A188" s="12"/>
+      <c r="B188" s="12"/>
       <c r="C188" s="1" t="s">
         <v>24</v>
       </c>
@@ -3798,14 +3799,14 @@
       <c r="E188" s="6">
         <v>74220</v>
       </c>
-      <c r="F188" s="9">
+      <c r="F188" s="11">
         <v>2968.8</v>
       </c>
-      <c r="G188" s="9"/>
+      <c r="G188" s="11"/>
     </row>
     <row r="189" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A189" s="10"/>
-      <c r="B189" s="10"/>
+      <c r="A189" s="12"/>
+      <c r="B189" s="12"/>
       <c r="C189" s="1" t="s">
         <v>25</v>
       </c>
@@ -3815,30 +3816,30 @@
       <c r="E189" s="6">
         <v>21250</v>
       </c>
-      <c r="F189" s="9">
+      <c r="F189" s="11">
         <v>2656.25</v>
       </c>
-      <c r="G189" s="9"/>
+      <c r="G189" s="11"/>
     </row>
     <row r="190" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A190" s="10"/>
-      <c r="B190" s="8" t="s">
+      <c r="A190" s="12"/>
+      <c r="B190" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C190" s="8"/>
+      <c r="C190" s="13"/>
       <c r="D190" s="5">
         <v>792</v>
       </c>
       <c r="E190" s="6">
         <v>2792340</v>
       </c>
-      <c r="F190" s="9">
+      <c r="F190" s="11">
         <v>3525.68</v>
       </c>
-      <c r="G190" s="9"/>
+      <c r="G190" s="11"/>
     </row>
     <row r="191" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A191" s="10"/>
+      <c r="A191" s="12"/>
       <c r="B191" s="4">
         <v>46292</v>
       </c>
@@ -3851,14 +3852,14 @@
       <c r="E191" s="6">
         <v>17550</v>
       </c>
-      <c r="F191" s="9">
+      <c r="F191" s="11">
         <v>4387.5</v>
       </c>
-      <c r="G191" s="9"/>
+      <c r="G191" s="11"/>
     </row>
     <row r="192" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="10"/>
-      <c r="B192" s="10"/>
+      <c r="A192" s="12"/>
+      <c r="B192" s="12"/>
       <c r="C192" s="1" t="s">
         <v>12</v>
       </c>
@@ -3868,14 +3869,14 @@
       <c r="E192" s="6">
         <v>18050</v>
       </c>
-      <c r="F192" s="9">
+      <c r="F192" s="11">
         <v>3610</v>
       </c>
-      <c r="G192" s="9"/>
+      <c r="G192" s="11"/>
     </row>
     <row r="193" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A193" s="10"/>
-      <c r="B193" s="10"/>
+      <c r="A193" s="12"/>
+      <c r="B193" s="12"/>
       <c r="C193" s="1" t="s">
         <v>13</v>
       </c>
@@ -3885,14 +3886,14 @@
       <c r="E193" s="6">
         <v>77700</v>
       </c>
-      <c r="F193" s="9">
+      <c r="F193" s="11">
         <v>4089.47</v>
       </c>
-      <c r="G193" s="9"/>
+      <c r="G193" s="11"/>
     </row>
     <row r="194" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A194" s="10"/>
-      <c r="B194" s="10"/>
+      <c r="A194" s="12"/>
+      <c r="B194" s="12"/>
       <c r="C194" s="1" t="s">
         <v>14</v>
       </c>
@@ -3902,14 +3903,14 @@
       <c r="E194" s="6">
         <v>87730</v>
       </c>
-      <c r="F194" s="9">
+      <c r="F194" s="11">
         <v>3509.2</v>
       </c>
-      <c r="G194" s="9"/>
+      <c r="G194" s="11"/>
     </row>
     <row r="195" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A195" s="10"/>
-      <c r="B195" s="10"/>
+      <c r="A195" s="12"/>
+      <c r="B195" s="12"/>
       <c r="C195" s="1" t="s">
         <v>15</v>
       </c>
@@ -3919,14 +3920,14 @@
       <c r="E195" s="6">
         <v>190930</v>
       </c>
-      <c r="F195" s="9">
+      <c r="F195" s="11">
         <v>3818.6</v>
       </c>
-      <c r="G195" s="9"/>
+      <c r="G195" s="11"/>
     </row>
     <row r="196" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" s="10"/>
-      <c r="B196" s="10"/>
+      <c r="A196" s="12"/>
+      <c r="B196" s="12"/>
       <c r="C196" s="1" t="s">
         <v>16</v>
       </c>
@@ -3936,14 +3937,14 @@
       <c r="E196" s="6">
         <v>256350</v>
       </c>
-      <c r="F196" s="9">
+      <c r="F196" s="11">
         <v>3884.09</v>
       </c>
-      <c r="G196" s="9"/>
+      <c r="G196" s="11"/>
     </row>
     <row r="197" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" s="10"/>
-      <c r="B197" s="10"/>
+      <c r="A197" s="12"/>
+      <c r="B197" s="12"/>
       <c r="C197" s="1" t="s">
         <v>17</v>
       </c>
@@ -3953,14 +3954,14 @@
       <c r="E197" s="6">
         <v>273750</v>
       </c>
-      <c r="F197" s="9">
+      <c r="F197" s="11">
         <v>3465.19</v>
       </c>
-      <c r="G197" s="9"/>
+      <c r="G197" s="11"/>
     </row>
     <row r="198" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A198" s="10"/>
-      <c r="B198" s="10"/>
+      <c r="A198" s="12"/>
+      <c r="B198" s="12"/>
       <c r="C198" s="1" t="s">
         <v>18</v>
       </c>
@@ -3970,14 +3971,14 @@
       <c r="E198" s="6">
         <v>369900</v>
       </c>
-      <c r="F198" s="9">
+      <c r="F198" s="11">
         <v>3244.74</v>
       </c>
-      <c r="G198" s="9"/>
+      <c r="G198" s="11"/>
     </row>
     <row r="199" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" s="10"/>
-      <c r="B199" s="10"/>
+      <c r="A199" s="12"/>
+      <c r="B199" s="12"/>
       <c r="C199" s="1" t="s">
         <v>19</v>
       </c>
@@ -3987,14 +3988,14 @@
       <c r="E199" s="6">
         <v>292670</v>
       </c>
-      <c r="F199" s="9">
+      <c r="F199" s="11">
         <v>3658.38</v>
       </c>
-      <c r="G199" s="9"/>
+      <c r="G199" s="11"/>
     </row>
     <row r="200" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="10"/>
-      <c r="B200" s="10"/>
+      <c r="A200" s="12"/>
+      <c r="B200" s="12"/>
       <c r="C200" s="1" t="s">
         <v>20</v>
       </c>
@@ -4004,14 +4005,14 @@
       <c r="E200" s="6">
         <v>282420</v>
       </c>
-      <c r="F200" s="9">
+      <c r="F200" s="11">
         <v>3444.15</v>
       </c>
-      <c r="G200" s="9"/>
+      <c r="G200" s="11"/>
     </row>
     <row r="201" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A201" s="10"/>
-      <c r="B201" s="10"/>
+      <c r="A201" s="12"/>
+      <c r="B201" s="12"/>
       <c r="C201" s="1" t="s">
         <v>21</v>
       </c>
@@ -4021,14 +4022,14 @@
       <c r="E201" s="6">
         <v>319190</v>
       </c>
-      <c r="F201" s="9">
+      <c r="F201" s="11">
         <v>3755.18</v>
       </c>
-      <c r="G201" s="9"/>
+      <c r="G201" s="11"/>
     </row>
     <row r="202" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="10"/>
-      <c r="B202" s="10"/>
+      <c r="A202" s="12"/>
+      <c r="B202" s="12"/>
       <c r="C202" s="1" t="s">
         <v>22</v>
       </c>
@@ -4038,14 +4039,14 @@
       <c r="E202" s="6">
         <v>211100</v>
       </c>
-      <c r="F202" s="9">
+      <c r="F202" s="11">
         <v>4139.22</v>
       </c>
-      <c r="G202" s="9"/>
+      <c r="G202" s="11"/>
     </row>
     <row r="203" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A203" s="10"/>
-      <c r="B203" s="10"/>
+      <c r="A203" s="12"/>
+      <c r="B203" s="12"/>
       <c r="C203" s="1" t="s">
         <v>23</v>
       </c>
@@ -4055,14 +4056,14 @@
       <c r="E203" s="6">
         <v>135500</v>
       </c>
-      <c r="F203" s="9">
+      <c r="F203" s="11">
         <v>3387.5</v>
       </c>
-      <c r="G203" s="9"/>
+      <c r="G203" s="11"/>
     </row>
     <row r="204" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A204" s="10"/>
-      <c r="B204" s="10"/>
+      <c r="A204" s="12"/>
+      <c r="B204" s="12"/>
       <c r="C204" s="1" t="s">
         <v>24</v>
       </c>
@@ -4072,14 +4073,14 @@
       <c r="E204" s="6">
         <v>36950</v>
       </c>
-      <c r="F204" s="9">
+      <c r="F204" s="11">
         <v>4105.5600000000004</v>
       </c>
-      <c r="G204" s="9"/>
+      <c r="G204" s="11"/>
     </row>
     <row r="205" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A205" s="10"/>
-      <c r="B205" s="10"/>
+      <c r="A205" s="12"/>
+      <c r="B205" s="12"/>
       <c r="C205" s="1" t="s">
         <v>25</v>
       </c>
@@ -4089,17 +4090,17 @@
       <c r="E205" s="6">
         <v>30750</v>
       </c>
-      <c r="F205" s="9">
+      <c r="F205" s="11">
         <v>2562.5</v>
       </c>
-      <c r="G205" s="9"/>
+      <c r="G205" s="11"/>
     </row>
     <row r="206" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A206" s="10"/>
-      <c r="B206" s="8" t="s">
+      <c r="A206" s="12"/>
+      <c r="B206" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C206" s="8"/>
+      <c r="C206" s="13"/>
       <c r="D206" s="5">
         <f>SUM(D191,D205)</f>
         <v>16</v>
@@ -4107,30 +4108,241 @@
       <c r="E206" s="6">
         <v>2600540</v>
       </c>
-      <c r="F206" s="9">
+      <c r="F206" s="11">
         <v>3606.85</v>
       </c>
-      <c r="G206" s="9"/>
+      <c r="G206" s="11"/>
     </row>
     <row r="207" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A207" s="8" t="s">
+      <c r="A207" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B207" s="8"/>
-      <c r="C207" s="8"/>
+      <c r="B207" s="13"/>
+      <c r="C207" s="13"/>
       <c r="D207" s="5">
         <v>6759</v>
       </c>
       <c r="E207" s="6">
         <v>23195780</v>
       </c>
-      <c r="F207" s="9">
+      <c r="F207" s="11">
         <v>3428.96</v>
       </c>
-      <c r="G207" s="9"/>
+      <c r="G207" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="235">
+    <mergeCell ref="B206:C206"/>
+    <mergeCell ref="F206:G206"/>
+    <mergeCell ref="A207:C207"/>
+    <mergeCell ref="F207:G207"/>
+    <mergeCell ref="B190:C190"/>
+    <mergeCell ref="F190:G190"/>
+    <mergeCell ref="F191:G191"/>
+    <mergeCell ref="B192:B205"/>
+    <mergeCell ref="F192:G192"/>
+    <mergeCell ref="F193:G193"/>
+    <mergeCell ref="F194:G194"/>
+    <mergeCell ref="F195:G195"/>
+    <mergeCell ref="F196:G196"/>
+    <mergeCell ref="F197:G197"/>
+    <mergeCell ref="F198:G198"/>
+    <mergeCell ref="F199:G199"/>
+    <mergeCell ref="F200:G200"/>
+    <mergeCell ref="F201:G201"/>
+    <mergeCell ref="F202:G202"/>
+    <mergeCell ref="F203:G203"/>
+    <mergeCell ref="F204:G204"/>
+    <mergeCell ref="F205:G205"/>
+    <mergeCell ref="B175:C175"/>
+    <mergeCell ref="F175:G175"/>
+    <mergeCell ref="F176:G176"/>
+    <mergeCell ref="B177:B189"/>
+    <mergeCell ref="F177:G177"/>
+    <mergeCell ref="F178:G178"/>
+    <mergeCell ref="F179:G179"/>
+    <mergeCell ref="F180:G180"/>
+    <mergeCell ref="F181:G181"/>
+    <mergeCell ref="F182:G182"/>
+    <mergeCell ref="F183:G183"/>
+    <mergeCell ref="F184:G184"/>
+    <mergeCell ref="F185:G185"/>
+    <mergeCell ref="F186:G186"/>
+    <mergeCell ref="F187:G187"/>
+    <mergeCell ref="F188:G188"/>
+    <mergeCell ref="F189:G189"/>
+    <mergeCell ref="B159:C159"/>
+    <mergeCell ref="F159:G159"/>
+    <mergeCell ref="F160:G160"/>
+    <mergeCell ref="F161:G161"/>
+    <mergeCell ref="B162:B174"/>
+    <mergeCell ref="F162:G162"/>
+    <mergeCell ref="F163:G163"/>
+    <mergeCell ref="F164:G164"/>
+    <mergeCell ref="F165:G165"/>
+    <mergeCell ref="F166:G166"/>
+    <mergeCell ref="F167:G167"/>
+    <mergeCell ref="F168:G168"/>
+    <mergeCell ref="F169:G169"/>
+    <mergeCell ref="F170:G170"/>
+    <mergeCell ref="F171:G171"/>
+    <mergeCell ref="F172:G172"/>
+    <mergeCell ref="F173:G173"/>
+    <mergeCell ref="F174:G174"/>
+    <mergeCell ref="B148:C148"/>
+    <mergeCell ref="F148:G148"/>
+    <mergeCell ref="F149:G149"/>
+    <mergeCell ref="B150:B158"/>
+    <mergeCell ref="F150:G150"/>
+    <mergeCell ref="F151:G151"/>
+    <mergeCell ref="F152:G152"/>
+    <mergeCell ref="F153:G153"/>
+    <mergeCell ref="F154:G154"/>
+    <mergeCell ref="F155:G155"/>
+    <mergeCell ref="F156:G156"/>
+    <mergeCell ref="F157:G157"/>
+    <mergeCell ref="F158:G158"/>
+    <mergeCell ref="B132:C132"/>
+    <mergeCell ref="F132:G132"/>
+    <mergeCell ref="F133:G133"/>
+    <mergeCell ref="B134:B147"/>
+    <mergeCell ref="F134:G134"/>
+    <mergeCell ref="F135:G135"/>
+    <mergeCell ref="F136:G136"/>
+    <mergeCell ref="F137:G137"/>
+    <mergeCell ref="F138:G138"/>
+    <mergeCell ref="F139:G139"/>
+    <mergeCell ref="F140:G140"/>
+    <mergeCell ref="F141:G141"/>
+    <mergeCell ref="F142:G142"/>
+    <mergeCell ref="F143:G143"/>
+    <mergeCell ref="F144:G144"/>
+    <mergeCell ref="F145:G145"/>
+    <mergeCell ref="F146:G146"/>
+    <mergeCell ref="F147:G147"/>
+    <mergeCell ref="B117:C117"/>
+    <mergeCell ref="F117:G117"/>
+    <mergeCell ref="F118:G118"/>
+    <mergeCell ref="B119:B131"/>
+    <mergeCell ref="F119:G119"/>
+    <mergeCell ref="F120:G120"/>
+    <mergeCell ref="F121:G121"/>
+    <mergeCell ref="F122:G122"/>
+    <mergeCell ref="F123:G123"/>
+    <mergeCell ref="F124:G124"/>
+    <mergeCell ref="F125:G125"/>
+    <mergeCell ref="F126:G126"/>
+    <mergeCell ref="F127:G127"/>
+    <mergeCell ref="F128:G128"/>
+    <mergeCell ref="F129:G129"/>
+    <mergeCell ref="F130:G130"/>
+    <mergeCell ref="F131:G131"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="F101:G101"/>
+    <mergeCell ref="F102:G102"/>
+    <mergeCell ref="B103:B116"/>
+    <mergeCell ref="F103:G103"/>
+    <mergeCell ref="F104:G104"/>
+    <mergeCell ref="F105:G105"/>
+    <mergeCell ref="F106:G106"/>
+    <mergeCell ref="F107:G107"/>
+    <mergeCell ref="F108:G108"/>
+    <mergeCell ref="F109:G109"/>
+    <mergeCell ref="F110:G110"/>
+    <mergeCell ref="F111:G111"/>
+    <mergeCell ref="F112:G112"/>
+    <mergeCell ref="F113:G113"/>
+    <mergeCell ref="F114:G114"/>
+    <mergeCell ref="F115:G115"/>
+    <mergeCell ref="F116:G116"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="F85:G85"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="B87:B100"/>
+    <mergeCell ref="F87:G87"/>
+    <mergeCell ref="F88:G88"/>
+    <mergeCell ref="F89:G89"/>
+    <mergeCell ref="F90:G90"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="F92:G92"/>
+    <mergeCell ref="F93:G93"/>
+    <mergeCell ref="F94:G94"/>
+    <mergeCell ref="F95:G95"/>
+    <mergeCell ref="F96:G96"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="F98:G98"/>
+    <mergeCell ref="F99:G99"/>
+    <mergeCell ref="F100:G100"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="B71:B84"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="B55:B68"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="B39:B52"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B23:B36"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
@@ -4155,217 +4367,6 @@
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B23:B36"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="B39:B52"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="B55:B68"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="B71:B84"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="F86:G86"/>
-    <mergeCell ref="B87:B100"/>
-    <mergeCell ref="F87:G87"/>
-    <mergeCell ref="F88:G88"/>
-    <mergeCell ref="F89:G89"/>
-    <mergeCell ref="F90:G90"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="F92:G92"/>
-    <mergeCell ref="F93:G93"/>
-    <mergeCell ref="F94:G94"/>
-    <mergeCell ref="F95:G95"/>
-    <mergeCell ref="F96:G96"/>
-    <mergeCell ref="F97:G97"/>
-    <mergeCell ref="F98:G98"/>
-    <mergeCell ref="F99:G99"/>
-    <mergeCell ref="F100:G100"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="F101:G101"/>
-    <mergeCell ref="F102:G102"/>
-    <mergeCell ref="B103:B116"/>
-    <mergeCell ref="F103:G103"/>
-    <mergeCell ref="F104:G104"/>
-    <mergeCell ref="F105:G105"/>
-    <mergeCell ref="F106:G106"/>
-    <mergeCell ref="F107:G107"/>
-    <mergeCell ref="F108:G108"/>
-    <mergeCell ref="F109:G109"/>
-    <mergeCell ref="F110:G110"/>
-    <mergeCell ref="F111:G111"/>
-    <mergeCell ref="F112:G112"/>
-    <mergeCell ref="F113:G113"/>
-    <mergeCell ref="F114:G114"/>
-    <mergeCell ref="F115:G115"/>
-    <mergeCell ref="F116:G116"/>
-    <mergeCell ref="B117:C117"/>
-    <mergeCell ref="F117:G117"/>
-    <mergeCell ref="F118:G118"/>
-    <mergeCell ref="B119:B131"/>
-    <mergeCell ref="F119:G119"/>
-    <mergeCell ref="F120:G120"/>
-    <mergeCell ref="F121:G121"/>
-    <mergeCell ref="F122:G122"/>
-    <mergeCell ref="F123:G123"/>
-    <mergeCell ref="F124:G124"/>
-    <mergeCell ref="F125:G125"/>
-    <mergeCell ref="F126:G126"/>
-    <mergeCell ref="F127:G127"/>
-    <mergeCell ref="F128:G128"/>
-    <mergeCell ref="F129:G129"/>
-    <mergeCell ref="F130:G130"/>
-    <mergeCell ref="F131:G131"/>
-    <mergeCell ref="B132:C132"/>
-    <mergeCell ref="F132:G132"/>
-    <mergeCell ref="F133:G133"/>
-    <mergeCell ref="B134:B147"/>
-    <mergeCell ref="F134:G134"/>
-    <mergeCell ref="F135:G135"/>
-    <mergeCell ref="F136:G136"/>
-    <mergeCell ref="F137:G137"/>
-    <mergeCell ref="F138:G138"/>
-    <mergeCell ref="F139:G139"/>
-    <mergeCell ref="F140:G140"/>
-    <mergeCell ref="F141:G141"/>
-    <mergeCell ref="F142:G142"/>
-    <mergeCell ref="F143:G143"/>
-    <mergeCell ref="F144:G144"/>
-    <mergeCell ref="F145:G145"/>
-    <mergeCell ref="F146:G146"/>
-    <mergeCell ref="F147:G147"/>
-    <mergeCell ref="B148:C148"/>
-    <mergeCell ref="F148:G148"/>
-    <mergeCell ref="F149:G149"/>
-    <mergeCell ref="B150:B158"/>
-    <mergeCell ref="F150:G150"/>
-    <mergeCell ref="F151:G151"/>
-    <mergeCell ref="F152:G152"/>
-    <mergeCell ref="F153:G153"/>
-    <mergeCell ref="F154:G154"/>
-    <mergeCell ref="F155:G155"/>
-    <mergeCell ref="F156:G156"/>
-    <mergeCell ref="F157:G157"/>
-    <mergeCell ref="F158:G158"/>
-    <mergeCell ref="B159:C159"/>
-    <mergeCell ref="F159:G159"/>
-    <mergeCell ref="F160:G160"/>
-    <mergeCell ref="F161:G161"/>
-    <mergeCell ref="B162:B174"/>
-    <mergeCell ref="F162:G162"/>
-    <mergeCell ref="F163:G163"/>
-    <mergeCell ref="F164:G164"/>
-    <mergeCell ref="F165:G165"/>
-    <mergeCell ref="F166:G166"/>
-    <mergeCell ref="F167:G167"/>
-    <mergeCell ref="F168:G168"/>
-    <mergeCell ref="F169:G169"/>
-    <mergeCell ref="F170:G170"/>
-    <mergeCell ref="F171:G171"/>
-    <mergeCell ref="F172:G172"/>
-    <mergeCell ref="F173:G173"/>
-    <mergeCell ref="F174:G174"/>
-    <mergeCell ref="B175:C175"/>
-    <mergeCell ref="F175:G175"/>
-    <mergeCell ref="F176:G176"/>
-    <mergeCell ref="B177:B189"/>
-    <mergeCell ref="F177:G177"/>
-    <mergeCell ref="F178:G178"/>
-    <mergeCell ref="F179:G179"/>
-    <mergeCell ref="F180:G180"/>
-    <mergeCell ref="F181:G181"/>
-    <mergeCell ref="F182:G182"/>
-    <mergeCell ref="F183:G183"/>
-    <mergeCell ref="F184:G184"/>
-    <mergeCell ref="F185:G185"/>
-    <mergeCell ref="F186:G186"/>
-    <mergeCell ref="F187:G187"/>
-    <mergeCell ref="F188:G188"/>
-    <mergeCell ref="F189:G189"/>
-    <mergeCell ref="B206:C206"/>
-    <mergeCell ref="F206:G206"/>
-    <mergeCell ref="A207:C207"/>
-    <mergeCell ref="F207:G207"/>
-    <mergeCell ref="B190:C190"/>
-    <mergeCell ref="F190:G190"/>
-    <mergeCell ref="F191:G191"/>
-    <mergeCell ref="B192:B205"/>
-    <mergeCell ref="F192:G192"/>
-    <mergeCell ref="F193:G193"/>
-    <mergeCell ref="F194:G194"/>
-    <mergeCell ref="F195:G195"/>
-    <mergeCell ref="F196:G196"/>
-    <mergeCell ref="F197:G197"/>
-    <mergeCell ref="F198:G198"/>
-    <mergeCell ref="F199:G199"/>
-    <mergeCell ref="F200:G200"/>
-    <mergeCell ref="F201:G201"/>
-    <mergeCell ref="F202:G202"/>
-    <mergeCell ref="F203:G203"/>
-    <mergeCell ref="F204:G204"/>
-    <mergeCell ref="F205:G205"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>

</xml_diff>